<commit_message>
Cover Page for Template. Other Fixes like HR FLAG
</commit_message>
<xml_diff>
--- a/Stat_Template_DO_NOT_REMOVE.xlsx
+++ b/Stat_Template_DO_NOT_REMOVE.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\super\OneDrive\Documents\Python Projects\SluggersStatTracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D50B218C-075D-4A26-8DA5-63F179609F7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632D315F-85F6-4B88-A681-87A98ED0E3D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2070" yWindow="3090" windowWidth="21600" windowHeight="11970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Stats" sheetId="1" r:id="rId1"/>
-    <sheet name="Pitching" sheetId="2" r:id="rId2"/>
+    <sheet name="Game Info" sheetId="3" r:id="rId1"/>
+    <sheet name="Stats" sheetId="1" r:id="rId2"/>
+    <sheet name="Pitching" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="83">
   <si>
     <t>Team</t>
   </si>
@@ -211,6 +213,78 @@
   </si>
   <si>
     <t>Inherited Runs</t>
+  </si>
+  <si>
+    <t>VS</t>
+  </si>
+  <si>
+    <t>Player Type 2</t>
+  </si>
+  <si>
+    <t>Stadium - Time of Day</t>
+  </si>
+  <si>
+    <t>Innings - X</t>
+  </si>
+  <si>
+    <t>Scorechart</t>
+  </si>
+  <si>
+    <t>Away Team</t>
+  </si>
+  <si>
+    <t>Home Team</t>
+  </si>
+  <si>
+    <t>XX</t>
+  </si>
+  <si>
+    <t>Stars - On/Off</t>
+  </si>
+  <si>
+    <t>Mercy - On/Off</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Pos</t>
+  </si>
+  <si>
+    <t>T1Player 1</t>
+  </si>
+  <si>
+    <t>T1Player 2</t>
+  </si>
+  <si>
+    <t>T1Player 3</t>
+  </si>
+  <si>
+    <t>T1Player 4</t>
+  </si>
+  <si>
+    <t>T1Player 5</t>
+  </si>
+  <si>
+    <t>T1Player 6</t>
+  </si>
+  <si>
+    <t>T1Player 7</t>
+  </si>
+  <si>
+    <t>T1Player 8</t>
+  </si>
+  <si>
+    <t>T1Player 9</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Items - On/Off</t>
+  </si>
+  <si>
+    <t>Player Type 1</t>
   </si>
 </sst>
 </file>
@@ -220,7 +294,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -265,8 +339,49 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="48"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="36"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -300,6 +415,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDBCDFF"/>
+        <bgColor rgb="FFD9D2E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor rgb="FFD9D2E9"/>
       </patternFill>
     </fill>
@@ -374,11 +495,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -386,9 +513,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -397,7 +523,6 @@
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -409,6 +534,29 @@
     <xf numFmtId="164" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -417,7 +565,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -637,6 +805,292 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDB774F7-11BA-460B-B512-6366E109F27E}">
+  <dimension ref="I10:S32"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="11" max="11" width="9.140625" customWidth="1"/>
+    <col min="13" max="13" width="9.140625" customWidth="1"/>
+    <col min="15" max="16" width="9.140625" customWidth="1"/>
+    <col min="18" max="18" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="10" spans="9:19" ht="18" x14ac:dyDescent="0.25">
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="23"/>
+    </row>
+    <row r="11" spans="9:19" ht="59.25" x14ac:dyDescent="0.75">
+      <c r="J11" s="18"/>
+      <c r="L11" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="N11" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="P11" s="17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="9:19" ht="40.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="I12" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="J12" s="29"/>
+      <c r="K12" s="29"/>
+      <c r="L12" s="29"/>
+      <c r="P12" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q12" s="29"/>
+      <c r="R12" s="29"/>
+      <c r="S12" s="29"/>
+    </row>
+    <row r="13" spans="9:19" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="I13" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="22"/>
+      <c r="P13" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q13" s="22"/>
+      <c r="R13" s="22"/>
+      <c r="S13" s="22"/>
+    </row>
+    <row r="14" spans="9:19" ht="18" x14ac:dyDescent="0.25">
+      <c r="I14" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
+      <c r="M14" s="23"/>
+      <c r="N14" s="23"/>
+      <c r="O14" s="23"/>
+      <c r="P14" s="23"/>
+      <c r="Q14" s="23"/>
+      <c r="R14" s="23"/>
+      <c r="S14" s="23"/>
+    </row>
+    <row r="15" spans="9:19" ht="18" x14ac:dyDescent="0.25">
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="N15" s="23"/>
+      <c r="O15" s="23"/>
+      <c r="P15" s="30"/>
+      <c r="Q15" s="30"/>
+      <c r="R15" s="30"/>
+      <c r="S15" s="30"/>
+    </row>
+    <row r="16" spans="9:19" ht="18" x14ac:dyDescent="0.25">
+      <c r="M16" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+    </row>
+    <row r="17" spans="10:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="M17" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+    </row>
+    <row r="18" spans="10:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="M18" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="N18" s="24"/>
+      <c r="O18" s="24"/>
+    </row>
+    <row r="19" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J19" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="K19" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q19" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="R19" s="31" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J20" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="K20" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q20" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="R20" s="35" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J21" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="K21" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q21" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="R21" s="35" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J22" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="K22" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q22" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="R22" s="35" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J23" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="K23" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q23" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="R23" s="35" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J24" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="K24" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q24" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="R24" s="35" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J25" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="K25" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q25" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="R25" s="35" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="26" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J26" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="K26" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q26" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="R26" s="35" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J27" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="K27" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q27" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="R27" s="35" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J28" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="K28" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q28" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="R28" s="35" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="29" spans="10:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="M29" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="N29" s="23"/>
+      <c r="O29" s="23"/>
+      <c r="P29" s="23"/>
+    </row>
+    <row r="31" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J31" s="21" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32" spans="10:18" ht="15" x14ac:dyDescent="0.2">
+      <c r="J32" s="21" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="L10:P10"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="M18:O18"/>
+    <mergeCell ref="I13:L13"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="P12:S12"/>
+    <mergeCell ref="I12:L12"/>
+    <mergeCell ref="I14:S14"/>
+    <mergeCell ref="M29:P29"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M16:O16"/>
+  </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -679,562 +1133,562 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8" t="s">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="P1" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="W1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="X1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="Y1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="Z1" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="AA1" s="9" t="s">
+      <c r="AA1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AB1" s="9" t="s">
+      <c r="AB1" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AC1" s="9" t="s">
+      <c r="AC1" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AD1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AE1" s="9" t="s">
+      <c r="AE1" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="AF1" s="10" t="s">
+      <c r="AF1" s="8" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="3"/>
-      <c r="T2" s="13"/>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="AF2" s="7"/>
+      <c r="F2" s="2"/>
+      <c r="T2" s="11"/>
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
+      <c r="AF2" s="6"/>
     </row>
     <row r="3" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="19"/>
-      <c r="B3" s="2" t="s">
+      <c r="A3" s="26"/>
+      <c r="B3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
-      <c r="AF3" s="7"/>
+      <c r="T3" s="11"/>
+      <c r="U3" s="11"/>
+      <c r="V3" s="11"/>
+      <c r="W3" s="11"/>
+      <c r="AF3" s="6"/>
     </row>
     <row r="4" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="19"/>
-      <c r="B4" s="2" t="s">
+      <c r="A4" s="26"/>
+      <c r="B4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M4" s="3"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="13"/>
-      <c r="V4" s="13"/>
-      <c r="W4" s="13"/>
-      <c r="AF4" s="7"/>
+      <c r="M4" s="2"/>
+      <c r="T4" s="11"/>
+      <c r="U4" s="11"/>
+      <c r="V4" s="11"/>
+      <c r="W4" s="11"/>
+      <c r="AF4" s="6"/>
     </row>
     <row r="5" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="19"/>
-      <c r="B5" s="2" t="s">
+      <c r="A5" s="26"/>
+      <c r="B5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="T5" s="13"/>
-      <c r="U5" s="13"/>
-      <c r="V5" s="13"/>
-      <c r="W5" s="13"/>
-      <c r="AF5" s="7"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="AF5" s="6"/>
     </row>
     <row r="6" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="19"/>
-      <c r="B6" s="2" t="s">
+      <c r="A6" s="26"/>
+      <c r="B6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="T6" s="13"/>
-      <c r="U6" s="13"/>
-      <c r="V6" s="13"/>
-      <c r="W6" s="13"/>
-      <c r="AF6" s="7"/>
+      <c r="T6" s="11"/>
+      <c r="U6" s="11"/>
+      <c r="V6" s="11"/>
+      <c r="W6" s="11"/>
+      <c r="AF6" s="6"/>
     </row>
     <row r="7" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="19"/>
-      <c r="B7" s="2" t="s">
+      <c r="A7" s="26"/>
+      <c r="B7" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="T7" s="13"/>
-      <c r="U7" s="13"/>
-      <c r="V7" s="13"/>
-      <c r="W7" s="13"/>
-      <c r="AF7" s="7"/>
+      <c r="T7" s="11"/>
+      <c r="U7" s="11"/>
+      <c r="V7" s="11"/>
+      <c r="W7" s="11"/>
+      <c r="AF7" s="6"/>
     </row>
     <row r="8" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="19"/>
-      <c r="B8" s="2" t="s">
+      <c r="A8" s="26"/>
+      <c r="B8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="T8" s="13"/>
-      <c r="U8" s="13"/>
-      <c r="V8" s="13"/>
-      <c r="W8" s="13"/>
-      <c r="AF8" s="7"/>
+      <c r="T8" s="11"/>
+      <c r="U8" s="11"/>
+      <c r="V8" s="11"/>
+      <c r="W8" s="11"/>
+      <c r="AF8" s="6"/>
     </row>
     <row r="9" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="19"/>
-      <c r="B9" s="2" t="s">
+      <c r="A9" s="26"/>
+      <c r="B9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="T9" s="13"/>
-      <c r="U9" s="13"/>
-      <c r="V9" s="13"/>
-      <c r="W9" s="13"/>
-      <c r="AF9" s="7"/>
+      <c r="T9" s="11"/>
+      <c r="U9" s="11"/>
+      <c r="V9" s="11"/>
+      <c r="W9" s="11"/>
+      <c r="AF9" s="6"/>
     </row>
     <row r="10" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="19"/>
-      <c r="B10" s="2" t="s">
+      <c r="A10" s="26"/>
+      <c r="B10" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="T10" s="13"/>
-      <c r="U10" s="13"/>
-      <c r="V10" s="13"/>
-      <c r="W10" s="13"/>
-      <c r="AF10" s="7"/>
+      <c r="T10" s="11"/>
+      <c r="U10" s="11"/>
+      <c r="V10" s="11"/>
+      <c r="W10" s="11"/>
+      <c r="AF10" s="6"/>
     </row>
     <row r="11" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="20"/>
-      <c r="B11" s="4" t="s">
+      <c r="A11" s="27"/>
+      <c r="B11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <f t="shared" ref="D11:S11" si="0">SUM(D2:D10)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K11" s="4">
+      <c r="K11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M11" s="4">
+      <c r="M11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N11" s="4">
+      <c r="N11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O11" s="4">
+      <c r="O11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P11" s="4">
+      <c r="P11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="Q11" s="4">
+      <c r="Q11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="R11" s="4">
+      <c r="R11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="S11" s="4">
+      <c r="S11" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T11" s="14">
+      <c r="T11" s="12">
         <f t="shared" ref="T11:W11" si="1">IFERROR(AVERAGE(T2:T10), 0)</f>
         <v>0</v>
       </c>
-      <c r="U11" s="14">
+      <c r="U11" s="12">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="V11" s="14">
+      <c r="V11" s="12">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="W11" s="14">
+      <c r="W11" s="12">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="X11" s="4">
+      <c r="X11" s="3">
         <f t="shared" ref="X11:AF11" si="2">SUM(X2:X10)</f>
         <v>0</v>
       </c>
-      <c r="Y11" s="4">
+      <c r="Y11" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Z11" s="4">
+      <c r="Z11" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AA11" s="4">
+      <c r="AA11" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AB11" s="4">
+      <c r="AB11" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AC11" s="4">
+      <c r="AC11" s="3">
         <f>SUM(AC2:AC10)</f>
         <v>0</v>
       </c>
-      <c r="AD11" s="4">
+      <c r="AD11" s="3">
         <f>SUM(AD2:AD10)</f>
         <v>0</v>
       </c>
-      <c r="AE11" s="4">
+      <c r="AE11" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AF11" s="4">
+      <c r="AF11" s="3">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="T12" s="13"/>
-      <c r="U12" s="13"/>
-      <c r="V12" s="13"/>
-      <c r="W12" s="13"/>
-      <c r="AF12" s="7"/>
+      <c r="T12" s="11"/>
+      <c r="U12" s="11"/>
+      <c r="V12" s="11"/>
+      <c r="W12" s="11"/>
+      <c r="AF12" s="6"/>
     </row>
     <row r="13" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="19"/>
-      <c r="B13" s="2" t="s">
+      <c r="A13" s="26"/>
+      <c r="B13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="T13" s="13"/>
-      <c r="U13" s="13"/>
-      <c r="V13" s="13"/>
-      <c r="W13" s="13"/>
-      <c r="AF13" s="7"/>
+      <c r="T13" s="11"/>
+      <c r="U13" s="11"/>
+      <c r="V13" s="11"/>
+      <c r="W13" s="11"/>
+      <c r="AF13" s="6"/>
     </row>
     <row r="14" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="19"/>
-      <c r="B14" s="2" t="s">
+      <c r="A14" s="26"/>
+      <c r="B14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="T14" s="13"/>
-      <c r="U14" s="13"/>
-      <c r="V14" s="13"/>
-      <c r="W14" s="13"/>
-      <c r="AF14" s="7"/>
+      <c r="T14" s="11"/>
+      <c r="U14" s="11"/>
+      <c r="V14" s="11"/>
+      <c r="W14" s="11"/>
+      <c r="AF14" s="6"/>
     </row>
     <row r="15" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="19"/>
-      <c r="B15" s="2" t="s">
+      <c r="A15" s="26"/>
+      <c r="B15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="T15" s="13"/>
-      <c r="U15" s="13"/>
-      <c r="V15" s="13"/>
-      <c r="W15" s="13"/>
-      <c r="AF15" s="7"/>
+      <c r="T15" s="11"/>
+      <c r="U15" s="11"/>
+      <c r="V15" s="11"/>
+      <c r="W15" s="11"/>
+      <c r="AF15" s="6"/>
     </row>
     <row r="16" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="19"/>
-      <c r="B16" s="2" t="s">
+      <c r="A16" s="26"/>
+      <c r="B16" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="T16" s="13"/>
-      <c r="U16" s="13"/>
-      <c r="V16" s="13"/>
-      <c r="W16" s="13"/>
-      <c r="AF16" s="7"/>
+      <c r="T16" s="11"/>
+      <c r="U16" s="11"/>
+      <c r="V16" s="11"/>
+      <c r="W16" s="11"/>
+      <c r="AF16" s="6"/>
     </row>
     <row r="17" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="19"/>
-      <c r="B17" s="2" t="s">
+      <c r="A17" s="26"/>
+      <c r="B17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="T17" s="13"/>
-      <c r="U17" s="13"/>
-      <c r="V17" s="13"/>
-      <c r="W17" s="13"/>
-      <c r="AF17" s="7"/>
+      <c r="T17" s="11"/>
+      <c r="U17" s="11"/>
+      <c r="V17" s="11"/>
+      <c r="W17" s="11"/>
+      <c r="AF17" s="6"/>
     </row>
     <row r="18" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="19"/>
-      <c r="B18" s="2" t="s">
+      <c r="A18" s="26"/>
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="T18" s="13"/>
-      <c r="U18" s="13"/>
-      <c r="V18" s="13"/>
-      <c r="W18" s="13"/>
-      <c r="AF18" s="7"/>
+      <c r="T18" s="11"/>
+      <c r="U18" s="11"/>
+      <c r="V18" s="11"/>
+      <c r="W18" s="11"/>
+      <c r="AF18" s="6"/>
     </row>
     <row r="19" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="19"/>
-      <c r="B19" s="2" t="s">
+      <c r="A19" s="26"/>
+      <c r="B19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="T19" s="13"/>
-      <c r="U19" s="13"/>
-      <c r="V19" s="13"/>
-      <c r="W19" s="13"/>
-      <c r="AF19" s="7"/>
+      <c r="T19" s="11"/>
+      <c r="U19" s="11"/>
+      <c r="V19" s="11"/>
+      <c r="W19" s="11"/>
+      <c r="AF19" s="6"/>
     </row>
     <row r="20" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="19"/>
-      <c r="B20" s="2" t="s">
+      <c r="A20" s="26"/>
+      <c r="B20" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="T20" s="13"/>
-      <c r="U20" s="13"/>
-      <c r="V20" s="13"/>
-      <c r="W20" s="13"/>
-      <c r="AF20" s="7"/>
+      <c r="T20" s="11"/>
+      <c r="U20" s="11"/>
+      <c r="V20" s="11"/>
+      <c r="W20" s="11"/>
+      <c r="AF20" s="6"/>
     </row>
     <row r="21" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="20"/>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="27"/>
+      <c r="B21" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="4">
         <f t="shared" ref="D21:S21" si="3">SUM(D12:D20)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K21" s="5">
+      <c r="K21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L21" s="5">
+      <c r="L21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M21" s="5">
+      <c r="M21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="N21" s="5">
+      <c r="N21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="O21" s="5">
+      <c r="O21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P21" s="5">
+      <c r="P21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="Q21" s="5">
+      <c r="Q21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="R21" s="5">
+      <c r="R21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S21" s="5">
+      <c r="S21" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="T21" s="15">
+      <c r="T21" s="13">
         <f t="shared" ref="T21:W21" si="4">IFERROR(AVERAGE(T12:T20), 0)</f>
         <v>0</v>
       </c>
-      <c r="U21" s="15">
+      <c r="U21" s="13">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="V21" s="15">
+      <c r="V21" s="13">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="W21" s="15">
+      <c r="W21" s="13">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="X21" s="5">
+      <c r="X21" s="4">
         <f t="shared" ref="X21:AF21" si="5">SUM(X12:X20)</f>
         <v>0</v>
       </c>
-      <c r="Y21" s="5">
+      <c r="Y21" s="4">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Z21" s="5">
+      <c r="Z21" s="4">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AA21" s="5">
+      <c r="AA21" s="4">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AB21" s="5">
+      <c r="AB21" s="4">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC21" s="5">
+      <c r="AC21" s="4">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AD21" s="5">
+      <c r="AD21" s="4">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AE21" s="5">
+      <c r="AE21" s="4">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AF21" s="5">
+      <c r="AF21" s="4">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="6"/>
+      <c r="A22" s="5"/>
     </row>
     <row r="29" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="9" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1247,7 +1701,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2">
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1260,339 +1714,339 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="36" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="12"/>
-      <c r="C2" s="17"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
+      <c r="A2" s="10"/>
+      <c r="C2" s="15"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
     </row>
     <row r="3" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="12"/>
-      <c r="C3" s="17"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
+      <c r="A3" s="10"/>
+      <c r="C3" s="15"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
     </row>
     <row r="4" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="12"/>
-      <c r="C4" s="17"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
+      <c r="A4" s="10"/>
+      <c r="C4" s="15"/>
+      <c r="O4" s="11"/>
+      <c r="P4" s="11"/>
+      <c r="Q4" s="11"/>
     </row>
     <row r="5" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="12"/>
-      <c r="C5" s="17"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
+      <c r="A5" s="10"/>
+      <c r="C5" s="15"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
     </row>
     <row r="6" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="12"/>
-      <c r="C6" s="17"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
+      <c r="A6" s="10"/>
+      <c r="C6" s="15"/>
+      <c r="O6" s="11"/>
+      <c r="P6" s="11"/>
+      <c r="Q6" s="11"/>
     </row>
     <row r="7" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="C7" s="17"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
+      <c r="A7" s="10"/>
+      <c r="C7" s="15"/>
+      <c r="O7" s="11"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11"/>
     </row>
     <row r="8" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="12"/>
-      <c r="C8" s="17"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="13"/>
-      <c r="Q8" s="13"/>
+      <c r="A8" s="10"/>
+      <c r="C8" s="15"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="11"/>
     </row>
     <row r="9" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="12"/>
-      <c r="C9" s="17"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="13"/>
+      <c r="A9" s="10"/>
+      <c r="C9" s="15"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="11"/>
     </row>
     <row r="10" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="12"/>
-      <c r="C10" s="17"/>
-      <c r="O10" s="13"/>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="13"/>
+      <c r="A10" s="10"/>
+      <c r="C10" s="15"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="11"/>
     </row>
     <row r="11" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="11"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="17"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
-      <c r="Q11" s="13"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="15"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="11"/>
     </row>
     <row r="12" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="11"/>
-      <c r="C12" s="17"/>
-      <c r="O12" s="13"/>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="13"/>
+      <c r="A12" s="9"/>
+      <c r="C12" s="15"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="11"/>
     </row>
     <row r="13" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="C13" s="17"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="13"/>
-      <c r="Q13" s="13"/>
+      <c r="A13" s="9"/>
+      <c r="C13" s="15"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="11"/>
+      <c r="Q13" s="11"/>
     </row>
     <row r="14" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="11"/>
-      <c r="C14" s="17"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="13"/>
+      <c r="A14" s="9"/>
+      <c r="C14" s="15"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="11"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="11"/>
-      <c r="C15" s="17"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="13"/>
+      <c r="A15" s="9"/>
+      <c r="C15" s="15"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="11"/>
+      <c r="Q15" s="11"/>
     </row>
     <row r="16" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="11"/>
-      <c r="C16" s="17"/>
-      <c r="O16" s="13"/>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="13"/>
+      <c r="A16" s="9"/>
+      <c r="C16" s="15"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="11"/>
+      <c r="Q16" s="11"/>
     </row>
     <row r="17" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="11"/>
-      <c r="C17" s="17"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="13"/>
+      <c r="A17" s="9"/>
+      <c r="C17" s="15"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="11"/>
+      <c r="Q17" s="11"/>
     </row>
     <row r="18" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="11"/>
-      <c r="C18" s="17"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="13"/>
+      <c r="A18" s="9"/>
+      <c r="C18" s="15"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="11"/>
+      <c r="Q18" s="11"/>
     </row>
     <row r="19" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="11"/>
-      <c r="C19" s="17"/>
-      <c r="O19" s="13"/>
-      <c r="P19" s="13"/>
-      <c r="Q19" s="13"/>
+      <c r="A19" s="9"/>
+      <c r="C19" s="15"/>
+      <c r="O19" s="11"/>
+      <c r="P19" s="11"/>
+      <c r="Q19" s="11"/>
     </row>
     <row r="20" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="11"/>
-      <c r="C20" s="17"/>
-      <c r="O20" s="13"/>
-      <c r="P20" s="13"/>
-      <c r="Q20" s="13"/>
+      <c r="A20" s="9"/>
+      <c r="C20" s="15"/>
+      <c r="O20" s="11"/>
+      <c r="P20" s="11"/>
+      <c r="Q20" s="11"/>
     </row>
     <row r="21" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="11"/>
-      <c r="C21" s="17"/>
-      <c r="O21" s="13"/>
-      <c r="P21" s="13"/>
-      <c r="Q21" s="13"/>
+      <c r="A21" s="9"/>
+      <c r="C21" s="15"/>
+      <c r="O21" s="11"/>
+      <c r="P21" s="11"/>
+      <c r="Q21" s="11"/>
     </row>
     <row r="22" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="11"/>
-      <c r="C22" s="17"/>
-      <c r="P22" s="13"/>
-      <c r="Q22" s="13"/>
+      <c r="A22" s="9"/>
+      <c r="C22" s="15"/>
+      <c r="P22" s="11"/>
+      <c r="Q22" s="11"/>
     </row>
     <row r="23" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="11"/>
-      <c r="C23" s="17"/>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="13"/>
+      <c r="A23" s="9"/>
+      <c r="C23" s="15"/>
+      <c r="P23" s="11"/>
+      <c r="Q23" s="11"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="11"/>
-      <c r="C24" s="17"/>
-      <c r="P24" s="13"/>
-      <c r="Q24" s="13"/>
+      <c r="A24" s="9"/>
+      <c r="C24" s="15"/>
+      <c r="P24" s="11"/>
+      <c r="Q24" s="11"/>
     </row>
     <row r="25" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="11"/>
-      <c r="C25" s="17"/>
-      <c r="P25" s="13"/>
-      <c r="Q25" s="13"/>
+      <c r="A25" s="9"/>
+      <c r="C25" s="15"/>
+      <c r="P25" s="11"/>
+      <c r="Q25" s="11"/>
     </row>
     <row r="26" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="11"/>
-      <c r="C26" s="17"/>
-      <c r="P26" s="13"/>
-      <c r="Q26" s="13"/>
+      <c r="A26" s="9"/>
+      <c r="C26" s="15"/>
+      <c r="P26" s="11"/>
+      <c r="Q26" s="11"/>
     </row>
     <row r="27" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C27" s="17"/>
-      <c r="P27" s="13"/>
-      <c r="Q27" s="13"/>
+      <c r="C27" s="15"/>
+      <c r="P27" s="11"/>
+      <c r="Q27" s="11"/>
     </row>
     <row r="28" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C28" s="17"/>
-      <c r="P28" s="13"/>
-      <c r="Q28" s="13"/>
+      <c r="C28" s="15"/>
+      <c r="P28" s="11"/>
+      <c r="Q28" s="11"/>
     </row>
     <row r="29" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C29" s="17"/>
-      <c r="P29" s="13"/>
-      <c r="Q29" s="13"/>
+      <c r="C29" s="15"/>
+      <c r="P29" s="11"/>
+      <c r="Q29" s="11"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C30" s="17"/>
-      <c r="P30" s="13"/>
-      <c r="Q30" s="13"/>
+      <c r="C30" s="15"/>
+      <c r="P30" s="11"/>
+      <c r="Q30" s="11"/>
     </row>
     <row r="31" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C31" s="17"/>
-      <c r="P31" s="13"/>
-      <c r="Q31" s="13"/>
+      <c r="C31" s="15"/>
+      <c r="P31" s="11"/>
+      <c r="Q31" s="11"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C32" s="17"/>
-      <c r="P32" s="13"/>
-      <c r="Q32" s="13"/>
+      <c r="C32" s="15"/>
+      <c r="P32" s="11"/>
+      <c r="Q32" s="11"/>
     </row>
     <row r="33" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C33" s="17"/>
-      <c r="P33" s="13"/>
-      <c r="Q33" s="13"/>
+      <c r="C33" s="15"/>
+      <c r="P33" s="11"/>
+      <c r="Q33" s="11"/>
     </row>
     <row r="34" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C34" s="17"/>
-      <c r="P34" s="13"/>
-      <c r="Q34" s="13"/>
+      <c r="C34" s="15"/>
+      <c r="P34" s="11"/>
+      <c r="Q34" s="11"/>
     </row>
     <row r="35" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C35" s="17"/>
-      <c r="P35" s="13"/>
-      <c r="Q35" s="13"/>
+      <c r="C35" s="15"/>
+      <c r="P35" s="11"/>
+      <c r="Q35" s="11"/>
     </row>
     <row r="36" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C36" s="17"/>
-      <c r="P36" s="13"/>
-      <c r="Q36" s="13"/>
+      <c r="C36" s="15"/>
+      <c r="P36" s="11"/>
+      <c r="Q36" s="11"/>
     </row>
     <row r="37" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C37" s="17"/>
-      <c r="P37" s="13"/>
-      <c r="Q37" s="13"/>
+      <c r="C37" s="15"/>
+      <c r="P37" s="11"/>
+      <c r="Q37" s="11"/>
     </row>
     <row r="38" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C38" s="17"/>
-      <c r="P38" s="13"/>
-      <c r="Q38" s="13"/>
+      <c r="C38" s="15"/>
+      <c r="P38" s="11"/>
+      <c r="Q38" s="11"/>
     </row>
     <row r="39" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C39" s="17"/>
+      <c r="C39" s="15"/>
     </row>
     <row r="40" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C40" s="17"/>
+      <c r="C40" s="15"/>
     </row>
     <row r="41" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C41" s="17"/>
+      <c r="C41" s="15"/>
     </row>
     <row r="42" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C42" s="17"/>
+      <c r="C42" s="15"/>
     </row>
     <row r="43" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C43" s="17"/>
+      <c r="C43" s="15"/>
     </row>
     <row r="44" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C44" s="17"/>
+      <c r="C44" s="15"/>
     </row>
     <row r="45" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C45" s="17"/>
+      <c r="C45" s="15"/>
     </row>
     <row r="46" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C46" s="17"/>
+      <c r="C46" s="15"/>
     </row>
     <row r="47" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C47" s="17"/>
+      <c r="C47" s="15"/>
     </row>
     <row r="48" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C48" s="17"/>
+      <c r="C48" s="15"/>
     </row>
     <row r="49" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C49" s="17"/>
+      <c r="C49" s="15"/>
     </row>
     <row r="50" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C50" s="17"/>
+      <c r="C50" s="15"/>
     </row>
     <row r="51" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C51" s="17"/>
+      <c r="C51" s="15"/>
     </row>
     <row r="52" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C52" s="17"/>
+      <c r="C52" s="15"/>
     </row>
     <row r="53" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C53" s="17"/>
+      <c r="C53" s="15"/>
     </row>
     <row r="54" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C54" s="17"/>
+      <c r="C54" s="15"/>
     </row>
     <row r="55" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C55" s="17"/>
+      <c r="C55" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
improved logging, expanded pitcher tracking, added back buddyjump tracking, changed template sheet
</commit_message>
<xml_diff>
--- a/Stat_Template_DO_NOT_REMOVE.xlsx
+++ b/Stat_Template_DO_NOT_REMOVE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\super\OneDrive\Documents\Python Projects\SluggersStatTracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632D315F-85F6-4B88-A681-87A98ED0E3D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F23BD0D5-8038-4AAA-9480-B85E07653AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game Info" sheetId="3" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="Pitching" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="93">
   <si>
     <t>Team</t>
   </si>
@@ -285,6 +284,36 @@
   </si>
   <si>
     <t>Player Type 1</t>
+  </si>
+  <si>
+    <t>Strikes</t>
+  </si>
+  <si>
+    <t>Balls</t>
+  </si>
+  <si>
+    <t>Pitches</t>
+  </si>
+  <si>
+    <t>Singles Allowed</t>
+  </si>
+  <si>
+    <t>Doubles Allowed</t>
+  </si>
+  <si>
+    <t>Triples Allowed</t>
+  </si>
+  <si>
+    <t>BA Against</t>
+  </si>
+  <si>
+    <t>OB% Against</t>
+  </si>
+  <si>
+    <t>SLG Against</t>
+  </si>
+  <si>
+    <t>OPS Against</t>
   </si>
 </sst>
 </file>
@@ -381,7 +410,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -415,12 +444,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDBCDFF"/>
-        <bgColor rgb="FFD9D2E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor rgb="FFD9D2E9"/>
       </patternFill>
     </fill>
@@ -513,7 +536,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -548,13 +571,24 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -565,27 +599,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -816,11 +830,11 @@
   </cols>
   <sheetData>
     <row r="10" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="23"/>
+      <c r="L10" s="26"/>
+      <c r="M10" s="26"/>
+      <c r="N10" s="26"/>
+      <c r="O10" s="26"/>
+      <c r="P10" s="26"/>
     </row>
     <row r="11" spans="9:19" ht="59.25" x14ac:dyDescent="0.75">
       <c r="J11" s="18"/>
@@ -849,217 +863,217 @@
       <c r="S12" s="29"/>
     </row>
     <row r="13" spans="9:19" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="I13" s="22" t="s">
+      <c r="I13" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="J13" s="22"/>
-      <c r="K13" s="22"/>
-      <c r="L13" s="22"/>
-      <c r="P13" s="22" t="s">
+      <c r="J13" s="28"/>
+      <c r="K13" s="28"/>
+      <c r="L13" s="28"/>
+      <c r="P13" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="Q13" s="22"/>
-      <c r="R13" s="22"/>
-      <c r="S13" s="22"/>
+      <c r="Q13" s="28"/>
+      <c r="R13" s="28"/>
+      <c r="S13" s="28"/>
     </row>
     <row r="14" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="I14" s="23" t="s">
+      <c r="I14" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="23"/>
-      <c r="P14" s="23"/>
-      <c r="Q14" s="23"/>
-      <c r="R14" s="23"/>
-      <c r="S14" s="23"/>
+      <c r="J14" s="26"/>
+      <c r="K14" s="26"/>
+      <c r="L14" s="26"/>
+      <c r="M14" s="26"/>
+      <c r="N14" s="26"/>
+      <c r="O14" s="26"/>
+      <c r="P14" s="26"/>
+      <c r="Q14" s="26"/>
+      <c r="R14" s="26"/>
+      <c r="S14" s="26"/>
     </row>
     <row r="15" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="I15" s="30"/>
-      <c r="J15" s="30"/>
-      <c r="K15" s="30"/>
-      <c r="L15" s="30"/>
-      <c r="M15" s="23" t="s">
+      <c r="I15" s="22"/>
+      <c r="J15" s="22"/>
+      <c r="K15" s="22"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="N15" s="23"/>
-      <c r="O15" s="23"/>
-      <c r="P15" s="30"/>
-      <c r="Q15" s="30"/>
-      <c r="R15" s="30"/>
-      <c r="S15" s="30"/>
+      <c r="N15" s="26"/>
+      <c r="O15" s="26"/>
+      <c r="P15" s="22"/>
+      <c r="Q15" s="22"/>
+      <c r="R15" s="22"/>
+      <c r="S15" s="22"/>
     </row>
     <row r="16" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="M16" s="23" t="s">
+      <c r="M16" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
+      <c r="N16" s="26"/>
+      <c r="O16" s="26"/>
     </row>
     <row r="17" spans="10:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="M17" s="23" t="s">
+      <c r="M17" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="N17" s="23"/>
-      <c r="O17" s="23"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="26"/>
     </row>
     <row r="18" spans="10:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="M18" s="23" t="s">
+      <c r="M18" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="N18" s="24"/>
-      <c r="O18" s="24"/>
+      <c r="N18" s="27"/>
+      <c r="O18" s="27"/>
     </row>
     <row r="19" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J19" s="31" t="s">
+      <c r="J19" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="K19" s="31" t="s">
+      <c r="K19" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="Q19" s="31" t="s">
+      <c r="Q19" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="R19" s="31" t="s">
+      <c r="R19" s="23" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="20" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J20" s="32" t="s">
+      <c r="J20" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="K20" s="33" t="s">
+      <c r="K20" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="Q20" s="33" t="s">
+      <c r="Q20" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="R20" s="35" t="s">
+      <c r="R20" s="24" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="21" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J21" s="32" t="s">
+      <c r="J21" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="K21" s="33" t="s">
+      <c r="K21" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="Q21" s="33" t="s">
+      <c r="Q21" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="R21" s="35" t="s">
+      <c r="R21" s="24" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="22" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J22" s="32" t="s">
+      <c r="J22" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="K22" s="34" t="s">
+      <c r="K22" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="Q22" s="34" t="s">
+      <c r="Q22" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="R22" s="35" t="s">
+      <c r="R22" s="24" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="23" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J23" s="32" t="s">
+      <c r="J23" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="K23" s="34" t="s">
+      <c r="K23" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="Q23" s="34" t="s">
+      <c r="Q23" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="R23" s="35" t="s">
+      <c r="R23" s="24" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="24" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J24" s="32" t="s">
+      <c r="J24" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="34" t="s">
+      <c r="K24" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="Q24" s="34" t="s">
+      <c r="Q24" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="R24" s="35" t="s">
+      <c r="R24" s="24" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="25" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J25" s="32" t="s">
+      <c r="J25" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="K25" s="34" t="s">
+      <c r="K25" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="Q25" s="34" t="s">
+      <c r="Q25" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="R25" s="35" t="s">
+      <c r="R25" s="24" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="26" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J26" s="32" t="s">
+      <c r="J26" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="K26" s="34" t="s">
+      <c r="K26" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="Q26" s="34" t="s">
+      <c r="Q26" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="R26" s="35" t="s">
+      <c r="R26" s="24" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="27" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J27" s="32" t="s">
+      <c r="J27" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="K27" s="34" t="s">
+      <c r="K27" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="Q27" s="34" t="s">
+      <c r="Q27" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="R27" s="35" t="s">
+      <c r="R27" s="24" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="28" spans="10:18" ht="15" x14ac:dyDescent="0.2">
-      <c r="J28" s="32" t="s">
+      <c r="J28" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="K28" s="34" t="s">
+      <c r="K28" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="Q28" s="34" t="s">
+      <c r="Q28" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="R28" s="35" t="s">
+      <c r="R28" s="24" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="29" spans="10:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="M29" s="23" t="s">
+      <c r="M29" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="N29" s="23"/>
-      <c r="O29" s="23"/>
-      <c r="P29" s="23"/>
+      <c r="N29" s="26"/>
+      <c r="O29" s="26"/>
+      <c r="P29" s="26"/>
     </row>
     <row r="31" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J31" s="21" t="s">
@@ -1073,6 +1087,9 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="M29:P29"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M16:O16"/>
     <mergeCell ref="L10:P10"/>
     <mergeCell ref="M17:O17"/>
     <mergeCell ref="M18:O18"/>
@@ -1081,9 +1098,6 @@
     <mergeCell ref="P12:S12"/>
     <mergeCell ref="I12:L12"/>
     <mergeCell ref="I14:S14"/>
-    <mergeCell ref="M29:P29"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="M16:O16"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1217,7 +1231,7 @@
       <c r="AB1" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AC1" s="37" t="s">
+      <c r="AC1" s="34" t="s">
         <v>52</v>
       </c>
       <c r="AD1" s="7" t="s">
@@ -1231,7 +1245,7 @@
       </c>
     </row>
     <row r="2" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="30" t="s">
         <v>28</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1245,7 +1259,7 @@
       <c r="AF2" s="6"/>
     </row>
     <row r="3" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="26"/>
+      <c r="A3" s="31"/>
       <c r="B3" s="1" t="s">
         <v>30</v>
       </c>
@@ -1256,7 +1270,7 @@
       <c r="AF3" s="6"/>
     </row>
     <row r="4" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="26"/>
+      <c r="A4" s="31"/>
       <c r="B4" s="1" t="s">
         <v>31</v>
       </c>
@@ -1268,7 +1282,7 @@
       <c r="AF4" s="6"/>
     </row>
     <row r="5" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="26"/>
+      <c r="A5" s="31"/>
       <c r="B5" s="1" t="s">
         <v>32</v>
       </c>
@@ -1279,7 +1293,7 @@
       <c r="AF5" s="6"/>
     </row>
     <row r="6" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="26"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="1" t="s">
         <v>33</v>
       </c>
@@ -1290,7 +1304,7 @@
       <c r="AF6" s="6"/>
     </row>
     <row r="7" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="26"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="1" t="s">
         <v>34</v>
       </c>
@@ -1301,7 +1315,7 @@
       <c r="AF7" s="6"/>
     </row>
     <row r="8" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="26"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="1" t="s">
         <v>35</v>
       </c>
@@ -1312,7 +1326,7 @@
       <c r="AF8" s="6"/>
     </row>
     <row r="9" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="26"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="1" t="s">
         <v>36</v>
       </c>
@@ -1323,7 +1337,7 @@
       <c r="AF9" s="6"/>
     </row>
     <row r="10" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="26"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="1" t="s">
         <v>37</v>
       </c>
@@ -1334,7 +1348,7 @@
       <c r="AF10" s="6"/>
     </row>
     <row r="11" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="27"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="3" t="s">
         <v>38</v>
       </c>
@@ -1459,7 +1473,7 @@
       </c>
     </row>
     <row r="12" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="33" t="s">
         <v>39</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -1472,7 +1486,7 @@
       <c r="AF12" s="6"/>
     </row>
     <row r="13" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="26"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="1" t="s">
         <v>30</v>
       </c>
@@ -1483,7 +1497,7 @@
       <c r="AF13" s="6"/>
     </row>
     <row r="14" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="26"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="1" t="s">
         <v>31</v>
       </c>
@@ -1494,7 +1508,7 @@
       <c r="AF14" s="6"/>
     </row>
     <row r="15" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="26"/>
+      <c r="A15" s="31"/>
       <c r="B15" s="1" t="s">
         <v>32</v>
       </c>
@@ -1505,7 +1519,7 @@
       <c r="AF15" s="6"/>
     </row>
     <row r="16" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="26"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="1" t="s">
         <v>33</v>
       </c>
@@ -1516,7 +1530,7 @@
       <c r="AF16" s="6"/>
     </row>
     <row r="17" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="26"/>
+      <c r="A17" s="31"/>
       <c r="B17" s="1" t="s">
         <v>34</v>
       </c>
@@ -1527,7 +1541,7 @@
       <c r="AF17" s="6"/>
     </row>
     <row r="18" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="26"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
@@ -1538,7 +1552,7 @@
       <c r="AF18" s="6"/>
     </row>
     <row r="19" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="26"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="1" t="s">
         <v>36</v>
       </c>
@@ -1549,7 +1563,7 @@
       <c r="AF19" s="6"/>
     </row>
     <row r="20" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="26"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="1" t="s">
         <v>37</v>
       </c>
@@ -1560,7 +1574,7 @@
       <c r="AF20" s="6"/>
     </row>
     <row r="21" spans="1:32" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="27"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="4" t="s">
         <v>38</v>
       </c>
@@ -1706,346 +1720,595 @@
   <sheetPr codeName="Sheet2">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:AA55"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="5" width="15.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" customWidth="1"/>
+    <col min="11" max="13" width="14.42578125" customWidth="1"/>
+    <col min="17" max="17" width="9" customWidth="1"/>
+    <col min="24" max="24" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="36" t="s">
+    <row r="1" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="36" t="s">
+      <c r="C1" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="I1" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="36" t="s">
+      <c r="J1" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="36" t="s">
+      <c r="K1" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="L1" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="M1" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="N1" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="36" t="s">
+      <c r="O1" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="36" t="s">
+      <c r="P1" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="K1" s="36" t="s">
+      <c r="Q1" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="36" t="s">
+      <c r="R1" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="M1" s="36" t="s">
+      <c r="S1" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="N1" s="36" t="s">
+      <c r="T1" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="O1" s="36" t="s">
+      <c r="U1" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="P1" s="36" t="s">
+      <c r="V1" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="Q1" s="36" t="s">
+      <c r="W1" s="25" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="X1" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y1" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z1" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA1" s="25" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="10"/>
       <c r="C2" s="15"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-    </row>
-    <row r="3" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+    </row>
+    <row r="3" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="10"/>
       <c r="C3" s="15"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-    </row>
-    <row r="4" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="U3" s="11"/>
+      <c r="V3" s="11"/>
+      <c r="W3" s="11"/>
+      <c r="X3" s="11"/>
+      <c r="Y3" s="11"/>
+      <c r="Z3" s="11"/>
+      <c r="AA3" s="11"/>
+    </row>
+    <row r="4" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="10"/>
       <c r="C4" s="15"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-    </row>
-    <row r="5" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="U4" s="11"/>
+      <c r="V4" s="11"/>
+      <c r="W4" s="11"/>
+      <c r="X4" s="11"/>
+      <c r="Y4" s="11"/>
+      <c r="Z4" s="11"/>
+      <c r="AA4" s="11"/>
+    </row>
+    <row r="5" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="10"/>
       <c r="C5" s="15"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-    </row>
-    <row r="6" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="U5" s="16"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
+      <c r="Y5" s="11"/>
+      <c r="Z5" s="11"/>
+      <c r="AA5" s="11"/>
+    </row>
+    <row r="6" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="10"/>
       <c r="C6" s="15"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-    </row>
-    <row r="7" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="U6" s="11"/>
+      <c r="V6" s="11"/>
+      <c r="W6" s="11"/>
+      <c r="X6" s="11"/>
+      <c r="Y6" s="11"/>
+      <c r="Z6" s="11"/>
+      <c r="AA6" s="11"/>
+    </row>
+    <row r="7" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="10"/>
       <c r="C7" s="15"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-    </row>
-    <row r="8" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="U7" s="11"/>
+      <c r="V7" s="11"/>
+      <c r="W7" s="11"/>
+      <c r="X7" s="11"/>
+      <c r="Y7" s="11"/>
+      <c r="Z7" s="11"/>
+      <c r="AA7" s="11"/>
+    </row>
+    <row r="8" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="10"/>
       <c r="C8" s="15"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-    </row>
-    <row r="9" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="U8" s="11"/>
+      <c r="V8" s="11"/>
+      <c r="W8" s="11"/>
+      <c r="X8" s="11"/>
+      <c r="Y8" s="11"/>
+      <c r="Z8" s="11"/>
+      <c r="AA8" s="11"/>
+    </row>
+    <row r="9" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="10"/>
       <c r="C9" s="15"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="11"/>
-    </row>
-    <row r="10" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="U9" s="11"/>
+      <c r="V9" s="11"/>
+      <c r="W9" s="11"/>
+      <c r="X9" s="11"/>
+      <c r="Y9" s="11"/>
+      <c r="Z9" s="11"/>
+      <c r="AA9" s="11"/>
+    </row>
+    <row r="10" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="10"/>
       <c r="C10" s="15"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="11"/>
-    </row>
-    <row r="11" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="U10" s="11"/>
+      <c r="V10" s="11"/>
+      <c r="W10" s="11"/>
+      <c r="X10" s="11"/>
+      <c r="Y10" s="11"/>
+      <c r="Z10" s="11"/>
+      <c r="AA10" s="11"/>
+    </row>
+    <row r="11" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="2"/>
       <c r="C11" s="15"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
-    </row>
-    <row r="12" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U11" s="11"/>
+      <c r="V11" s="11"/>
+      <c r="W11" s="11"/>
+      <c r="X11" s="11"/>
+      <c r="Y11" s="11"/>
+      <c r="Z11" s="11"/>
+      <c r="AA11" s="11"/>
+    </row>
+    <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="C12" s="15"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
-    </row>
-    <row r="13" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U12" s="11"/>
+      <c r="V12" s="11"/>
+      <c r="W12" s="11"/>
+      <c r="X12" s="11"/>
+      <c r="Y12" s="11"/>
+      <c r="Z12" s="11"/>
+      <c r="AA12" s="11"/>
+    </row>
+    <row r="13" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9"/>
       <c r="C13" s="15"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-    </row>
-    <row r="14" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U13" s="11"/>
+      <c r="V13" s="11"/>
+      <c r="W13" s="11"/>
+      <c r="X13" s="11"/>
+      <c r="Y13" s="11"/>
+      <c r="Z13" s="11"/>
+      <c r="AA13" s="11"/>
+    </row>
+    <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9"/>
       <c r="C14" s="15"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="11"/>
-    </row>
-    <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U14" s="11"/>
+      <c r="V14" s="11"/>
+      <c r="W14" s="11"/>
+      <c r="X14" s="11"/>
+      <c r="Y14" s="11"/>
+      <c r="Z14" s="11"/>
+      <c r="AA14" s="11"/>
+    </row>
+    <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9"/>
       <c r="C15" s="15"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="11"/>
-    </row>
-    <row r="16" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U15" s="11"/>
+      <c r="V15" s="11"/>
+      <c r="W15" s="11"/>
+      <c r="X15" s="11"/>
+      <c r="Y15" s="11"/>
+      <c r="Z15" s="11"/>
+      <c r="AA15" s="11"/>
+    </row>
+    <row r="16" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9"/>
       <c r="C16" s="15"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="11"/>
-    </row>
-    <row r="17" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U16" s="11"/>
+      <c r="V16" s="11"/>
+      <c r="W16" s="11"/>
+      <c r="X16" s="11"/>
+      <c r="Y16" s="11"/>
+      <c r="Z16" s="11"/>
+      <c r="AA16" s="11"/>
+    </row>
+    <row r="17" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9"/>
       <c r="C17" s="15"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="11"/>
-      <c r="Q17" s="11"/>
-    </row>
-    <row r="18" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U17" s="11"/>
+      <c r="V17" s="11"/>
+      <c r="W17" s="11"/>
+      <c r="X17" s="11"/>
+      <c r="Y17" s="11"/>
+      <c r="Z17" s="11"/>
+      <c r="AA17" s="11"/>
+    </row>
+    <row r="18" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="9"/>
       <c r="C18" s="15"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="11"/>
-    </row>
-    <row r="19" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U18" s="11"/>
+      <c r="V18" s="11"/>
+      <c r="W18" s="11"/>
+      <c r="X18" s="11"/>
+      <c r="Y18" s="11"/>
+      <c r="Z18" s="11"/>
+      <c r="AA18" s="11"/>
+    </row>
+    <row r="19" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="C19" s="15"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="11"/>
-    </row>
-    <row r="20" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U19" s="11"/>
+      <c r="V19" s="11"/>
+      <c r="W19" s="11"/>
+      <c r="X19" s="11"/>
+      <c r="Y19" s="11"/>
+      <c r="Z19" s="11"/>
+      <c r="AA19" s="11"/>
+    </row>
+    <row r="20" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="C20" s="15"/>
-      <c r="O20" s="11"/>
-      <c r="P20" s="11"/>
-      <c r="Q20" s="11"/>
-    </row>
-    <row r="21" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U20" s="11"/>
+      <c r="V20" s="11"/>
+      <c r="W20" s="11"/>
+      <c r="X20" s="11"/>
+      <c r="Y20" s="11"/>
+      <c r="Z20" s="11"/>
+      <c r="AA20" s="11"/>
+    </row>
+    <row r="21" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="C21" s="15"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="11"/>
-    </row>
-    <row r="22" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U21" s="11"/>
+      <c r="V21" s="11"/>
+      <c r="W21" s="11"/>
+      <c r="X21" s="11"/>
+      <c r="Y21" s="11"/>
+      <c r="Z21" s="11"/>
+      <c r="AA21" s="11"/>
+    </row>
+    <row r="22" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9"/>
       <c r="C22" s="15"/>
-      <c r="P22" s="11"/>
-      <c r="Q22" s="11"/>
-    </row>
-    <row r="23" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V22" s="11"/>
+      <c r="W22" s="11"/>
+      <c r="X22" s="11"/>
+      <c r="Y22" s="11"/>
+      <c r="Z22" s="11"/>
+      <c r="AA22" s="11"/>
+    </row>
+    <row r="23" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="C23" s="15"/>
-      <c r="P23" s="11"/>
-      <c r="Q23" s="11"/>
-    </row>
-    <row r="24" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V23" s="11"/>
+      <c r="W23" s="11"/>
+      <c r="X23" s="11"/>
+      <c r="Y23" s="11"/>
+      <c r="Z23" s="11"/>
+      <c r="AA23" s="11"/>
+    </row>
+    <row r="24" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9"/>
       <c r="C24" s="15"/>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="11"/>
-    </row>
-    <row r="25" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V24" s="11"/>
+      <c r="W24" s="11"/>
+      <c r="X24" s="11"/>
+      <c r="Y24" s="11"/>
+      <c r="Z24" s="11"/>
+      <c r="AA24" s="11"/>
+    </row>
+    <row r="25" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
       <c r="C25" s="15"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="11"/>
-    </row>
-    <row r="26" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V25" s="11"/>
+      <c r="W25" s="11"/>
+      <c r="X25" s="11"/>
+      <c r="Y25" s="11"/>
+      <c r="Z25" s="11"/>
+      <c r="AA25" s="11"/>
+    </row>
+    <row r="26" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="9"/>
       <c r="C26" s="15"/>
-      <c r="P26" s="11"/>
-      <c r="Q26" s="11"/>
-    </row>
-    <row r="27" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V26" s="11"/>
+      <c r="W26" s="11"/>
+      <c r="X26" s="11"/>
+      <c r="Y26" s="11"/>
+      <c r="Z26" s="11"/>
+      <c r="AA26" s="11"/>
+    </row>
+    <row r="27" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C27" s="15"/>
-      <c r="P27" s="11"/>
-      <c r="Q27" s="11"/>
-    </row>
-    <row r="28" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V27" s="11"/>
+      <c r="W27" s="11"/>
+      <c r="X27" s="11"/>
+      <c r="Y27" s="11"/>
+      <c r="Z27" s="11"/>
+      <c r="AA27" s="11"/>
+    </row>
+    <row r="28" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C28" s="15"/>
-      <c r="P28" s="11"/>
-      <c r="Q28" s="11"/>
-    </row>
-    <row r="29" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V28" s="11"/>
+      <c r="W28" s="11"/>
+      <c r="X28" s="11"/>
+      <c r="Y28" s="11"/>
+      <c r="Z28" s="11"/>
+      <c r="AA28" s="11"/>
+    </row>
+    <row r="29" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C29" s="15"/>
-      <c r="P29" s="11"/>
-      <c r="Q29" s="11"/>
-    </row>
-    <row r="30" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V29" s="11"/>
+      <c r="W29" s="11"/>
+      <c r="X29" s="11"/>
+      <c r="Y29" s="11"/>
+      <c r="Z29" s="11"/>
+      <c r="AA29" s="11"/>
+    </row>
+    <row r="30" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C30" s="15"/>
-      <c r="P30" s="11"/>
-      <c r="Q30" s="11"/>
-    </row>
-    <row r="31" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V30" s="11"/>
+      <c r="W30" s="11"/>
+      <c r="X30" s="11"/>
+      <c r="Y30" s="11"/>
+      <c r="Z30" s="11"/>
+      <c r="AA30" s="11"/>
+    </row>
+    <row r="31" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C31" s="15"/>
-      <c r="P31" s="11"/>
-      <c r="Q31" s="11"/>
-    </row>
-    <row r="32" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V31" s="11"/>
+      <c r="W31" s="11"/>
+      <c r="X31" s="11"/>
+      <c r="Y31" s="11"/>
+      <c r="Z31" s="11"/>
+      <c r="AA31" s="11"/>
+    </row>
+    <row r="32" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C32" s="15"/>
-      <c r="P32" s="11"/>
-      <c r="Q32" s="11"/>
-    </row>
-    <row r="33" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V32" s="11"/>
+      <c r="W32" s="11"/>
+      <c r="X32" s="11"/>
+      <c r="Y32" s="11"/>
+      <c r="Z32" s="11"/>
+      <c r="AA32" s="11"/>
+    </row>
+    <row r="33" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C33" s="15"/>
-      <c r="P33" s="11"/>
-      <c r="Q33" s="11"/>
-    </row>
-    <row r="34" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V33" s="11"/>
+      <c r="W33" s="11"/>
+      <c r="X33" s="11"/>
+      <c r="Y33" s="11"/>
+      <c r="Z33" s="11"/>
+      <c r="AA33" s="11"/>
+    </row>
+    <row r="34" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C34" s="15"/>
-      <c r="P34" s="11"/>
-      <c r="Q34" s="11"/>
-    </row>
-    <row r="35" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V34" s="11"/>
+      <c r="W34" s="11"/>
+      <c r="X34" s="11"/>
+      <c r="Y34" s="11"/>
+      <c r="Z34" s="11"/>
+      <c r="AA34" s="11"/>
+    </row>
+    <row r="35" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C35" s="15"/>
-      <c r="P35" s="11"/>
-      <c r="Q35" s="11"/>
-    </row>
-    <row r="36" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V35" s="11"/>
+      <c r="W35" s="11"/>
+      <c r="X35" s="11"/>
+      <c r="Y35" s="11"/>
+      <c r="Z35" s="11"/>
+      <c r="AA35" s="11"/>
+    </row>
+    <row r="36" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C36" s="15"/>
-      <c r="P36" s="11"/>
-      <c r="Q36" s="11"/>
-    </row>
-    <row r="37" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V36" s="11"/>
+      <c r="W36" s="11"/>
+      <c r="X36" s="11"/>
+      <c r="Y36" s="11"/>
+      <c r="Z36" s="11"/>
+      <c r="AA36" s="11"/>
+    </row>
+    <row r="37" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C37" s="15"/>
-      <c r="P37" s="11"/>
-      <c r="Q37" s="11"/>
-    </row>
-    <row r="38" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V37" s="11"/>
+      <c r="W37" s="11"/>
+      <c r="X37" s="11"/>
+      <c r="Y37" s="11"/>
+      <c r="Z37" s="11"/>
+      <c r="AA37" s="11"/>
+    </row>
+    <row r="38" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C38" s="15"/>
-      <c r="P38" s="11"/>
-      <c r="Q38" s="11"/>
-    </row>
-    <row r="39" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V38" s="11"/>
+      <c r="W38" s="11"/>
+      <c r="X38" s="11"/>
+      <c r="Y38" s="11"/>
+      <c r="Z38" s="11"/>
+      <c r="AA38" s="11"/>
+    </row>
+    <row r="39" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C39" s="15"/>
-    </row>
-    <row r="40" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X39" s="11"/>
+      <c r="Y39" s="11"/>
+      <c r="Z39" s="11"/>
+      <c r="AA39" s="11"/>
+    </row>
+    <row r="40" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C40" s="15"/>
-    </row>
-    <row r="41" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X40" s="11"/>
+      <c r="Y40" s="11"/>
+      <c r="Z40" s="11"/>
+      <c r="AA40" s="11"/>
+    </row>
+    <row r="41" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C41" s="15"/>
-    </row>
-    <row r="42" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X41" s="11"/>
+      <c r="Y41" s="11"/>
+      <c r="Z41" s="11"/>
+      <c r="AA41" s="11"/>
+    </row>
+    <row r="42" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C42" s="15"/>
-    </row>
-    <row r="43" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X42" s="11"/>
+      <c r="Y42" s="11"/>
+      <c r="Z42" s="11"/>
+      <c r="AA42" s="11"/>
+    </row>
+    <row r="43" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C43" s="15"/>
-    </row>
-    <row r="44" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X43" s="11"/>
+      <c r="Y43" s="11"/>
+      <c r="Z43" s="11"/>
+      <c r="AA43" s="11"/>
+    </row>
+    <row r="44" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C44" s="15"/>
-    </row>
-    <row r="45" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X44" s="11"/>
+      <c r="Y44" s="11"/>
+      <c r="Z44" s="11"/>
+      <c r="AA44" s="11"/>
+    </row>
+    <row r="45" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C45" s="15"/>
-    </row>
-    <row r="46" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X45" s="11"/>
+      <c r="Y45" s="11"/>
+      <c r="Z45" s="11"/>
+      <c r="AA45" s="11"/>
+    </row>
+    <row r="46" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C46" s="15"/>
-    </row>
-    <row r="47" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X46" s="11"/>
+      <c r="Y46" s="11"/>
+      <c r="Z46" s="11"/>
+      <c r="AA46" s="11"/>
+    </row>
+    <row r="47" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C47" s="15"/>
-    </row>
-    <row r="48" spans="3:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X47" s="11"/>
+      <c r="Y47" s="11"/>
+      <c r="Z47" s="11"/>
+      <c r="AA47" s="11"/>
+    </row>
+    <row r="48" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C48" s="15"/>
-    </row>
-    <row r="49" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X48" s="11"/>
+      <c r="Y48" s="11"/>
+      <c r="Z48" s="11"/>
+      <c r="AA48" s="11"/>
+    </row>
+    <row r="49" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C49" s="15"/>
-    </row>
-    <row r="50" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X49" s="11"/>
+      <c r="Y49" s="11"/>
+      <c r="Z49" s="11"/>
+      <c r="AA49" s="11"/>
+    </row>
+    <row r="50" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C50" s="15"/>
-    </row>
-    <row r="51" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X50" s="11"/>
+      <c r="Y50" s="11"/>
+      <c r="Z50" s="11"/>
+      <c r="AA50" s="11"/>
+    </row>
+    <row r="51" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C51" s="15"/>
-    </row>
-    <row r="52" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X51" s="11"/>
+      <c r="Y51" s="11"/>
+      <c r="Z51" s="11"/>
+      <c r="AA51" s="11"/>
+    </row>
+    <row r="52" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C52" s="15"/>
-    </row>
-    <row r="53" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X52" s="11"/>
+      <c r="Y52" s="11"/>
+      <c r="Z52" s="11"/>
+      <c r="AA52" s="11"/>
+    </row>
+    <row r="53" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C53" s="15"/>
-    </row>
-    <row r="54" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X53" s="11"/>
+      <c r="Y53" s="11"/>
+      <c r="Z53" s="11"/>
+      <c r="AA53" s="11"/>
+    </row>
+    <row r="54" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C54" s="15"/>
-    </row>
-    <row r="55" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X54" s="11"/>
+      <c r="Y54" s="11"/>
+      <c r="Z54" s="11"/>
+      <c r="AA54" s="11"/>
+    </row>
+    <row r="55" spans="3:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C55" s="15"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
massive refactor of outputter. changed team stat math.
</commit_message>
<xml_diff>
--- a/Stat_Template_DO_NOT_REMOVE.xlsx
+++ b/Stat_Template_DO_NOT_REMOVE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\super\OneDrive\Documents\Python Projects\SluggersStatTracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E90910C-E634-48A1-BF82-3AC2E883C57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59FA2570-89A2-4970-9A18-5A8ED2D0626D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-1950" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game Info" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="99">
   <si>
     <t>Team</t>
   </si>
@@ -182,9 +182,6 @@
   </si>
   <si>
     <t>Steal Attempts</t>
-  </si>
-  <si>
-    <t>RED = NOT BEING TRACKED YET</t>
   </si>
   <si>
     <t>Buddy Jump Putouts</t>
@@ -614,6 +611,18 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -625,18 +634,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -868,18 +865,18 @@
   </cols>
   <sheetData>
     <row r="9" spans="9:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="L9" s="30"/>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="30"/>
-      <c r="P9" s="30"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="34"/>
+      <c r="N9" s="34"/>
+      <c r="O9" s="34"/>
+      <c r="P9" s="34"/>
     </row>
     <row r="10" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="L10" s="31"/>
-      <c r="M10" s="31"/>
-      <c r="N10" s="31"/>
-      <c r="O10" s="31"/>
-      <c r="P10" s="31"/>
+      <c r="L10" s="35"/>
+      <c r="M10" s="35"/>
+      <c r="N10" s="35"/>
+      <c r="O10" s="35"/>
+      <c r="P10" s="35"/>
     </row>
     <row r="11" spans="9:19" ht="59.25" x14ac:dyDescent="0.75">
       <c r="J11" s="14"/>
@@ -887,247 +884,247 @@
         <v>27</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="P11" s="13" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="12" spans="9:19" ht="40.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="I12" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="J12" s="33"/>
-      <c r="K12" s="33"/>
-      <c r="L12" s="33"/>
-      <c r="P12" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q12" s="33"/>
-      <c r="R12" s="33"/>
-      <c r="S12" s="33"/>
+      <c r="I12" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="J12" s="37"/>
+      <c r="K12" s="37"/>
+      <c r="L12" s="37"/>
+      <c r="P12" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q12" s="37"/>
+      <c r="R12" s="37"/>
+      <c r="S12" s="37"/>
     </row>
     <row r="13" spans="9:19" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="I13" s="32" t="s">
-        <v>77</v>
-      </c>
-      <c r="J13" s="32"/>
-      <c r="K13" s="32"/>
-      <c r="L13" s="32"/>
-      <c r="P13" s="32" t="s">
+      <c r="I13" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="J13" s="36"/>
+      <c r="K13" s="36"/>
+      <c r="L13" s="36"/>
+      <c r="P13" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q13" s="36"/>
+      <c r="R13" s="36"/>
+      <c r="S13" s="36"/>
+    </row>
+    <row r="14" spans="9:19" ht="18" x14ac:dyDescent="0.25">
+      <c r="I14" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="Q13" s="32"/>
-      <c r="R13" s="32"/>
-      <c r="S13" s="32"/>
-    </row>
-    <row r="14" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="I14" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="31"/>
-      <c r="M14" s="31"/>
-      <c r="N14" s="31"/>
-      <c r="O14" s="31"/>
-      <c r="P14" s="31"/>
-      <c r="Q14" s="31"/>
-      <c r="R14" s="31"/>
-      <c r="S14" s="31"/>
+      <c r="J14" s="35"/>
+      <c r="K14" s="35"/>
+      <c r="L14" s="35"/>
+      <c r="M14" s="35"/>
+      <c r="N14" s="35"/>
+      <c r="O14" s="35"/>
+      <c r="P14" s="35"/>
+      <c r="Q14" s="35"/>
+      <c r="R14" s="35"/>
+      <c r="S14" s="35"/>
     </row>
     <row r="15" spans="9:19" ht="18" x14ac:dyDescent="0.25">
       <c r="I15" s="18"/>
       <c r="J15" s="18"/>
       <c r="K15" s="18"/>
       <c r="L15" s="18"/>
-      <c r="M15" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="N15" s="31"/>
-      <c r="O15" s="31"/>
+      <c r="M15" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="N15" s="35"/>
+      <c r="O15" s="35"/>
       <c r="P15" s="18"/>
       <c r="Q15" s="18"/>
       <c r="R15" s="18"/>
       <c r="S15" s="18"/>
     </row>
     <row r="16" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="M16" s="31" t="s">
-        <v>63</v>
-      </c>
-      <c r="N16" s="31"/>
-      <c r="O16" s="31"/>
+      <c r="M16" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="N16" s="35"/>
+      <c r="O16" s="35"/>
     </row>
     <row r="17" spans="10:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="M17" s="31" t="s">
-        <v>62</v>
-      </c>
-      <c r="N17" s="31"/>
-      <c r="O17" s="31"/>
+      <c r="M17" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="N17" s="35"/>
+      <c r="O17" s="35"/>
     </row>
     <row r="18" spans="10:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="M18" s="31" t="s">
-        <v>76</v>
-      </c>
-      <c r="N18" s="30"/>
-      <c r="O18" s="30"/>
+      <c r="M18" s="35" t="s">
+        <v>75</v>
+      </c>
+      <c r="N18" s="34"/>
+      <c r="O18" s="34"/>
     </row>
     <row r="19" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J19" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="K19" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="K19" s="19" t="s">
-        <v>65</v>
-      </c>
       <c r="Q19" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="R19" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J20" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K20" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q20" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R20" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J21" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K21" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q21" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R21" s="20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J22" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K22" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q22" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R22" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J23" s="17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K23" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q23" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R23" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J24" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K24" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q24" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R24" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J25" s="17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K25" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q25" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R25" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J26" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K26" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q26" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R26" s="20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J27" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K27" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q27" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R27" s="20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J28" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="K28" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="K28" s="19" t="s">
-        <v>75</v>
-      </c>
       <c r="Q28" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="R28" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="10:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="M29" s="31" t="s">
-        <v>89</v>
-      </c>
-      <c r="N29" s="31"/>
-      <c r="O29" s="31"/>
-      <c r="P29" s="31"/>
+      <c r="M29" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="N29" s="35"/>
+      <c r="O29" s="35"/>
+      <c r="P29" s="35"/>
     </row>
     <row r="31" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J31" s="17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J32" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1211,7 +1208,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F1" s="24" t="s">
         <v>4</v>
@@ -1244,16 +1241,16 @@
         <v>13</v>
       </c>
       <c r="P1" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q1" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="Q1" s="24" t="s">
+      <c r="R1" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="R1" s="24" t="s">
+      <c r="S1" s="24" t="s">
         <v>95</v>
-      </c>
-      <c r="S1" s="24" t="s">
-        <v>96</v>
       </c>
       <c r="T1" s="23" t="s">
         <v>14</v>
@@ -1262,13 +1259,13 @@
         <v>15</v>
       </c>
       <c r="V1" s="24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="W1" s="24" t="s">
         <v>16</v>
       </c>
       <c r="X1" s="24" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Y1" s="24" t="s">
         <v>17</v>
@@ -1283,7 +1280,7 @@
         <v>20</v>
       </c>
       <c r="AC1" s="24" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AD1" s="24" t="s">
         <v>21</v>
@@ -1301,10 +1298,10 @@
         <v>24</v>
       </c>
       <c r="AI1" s="24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AJ1" s="24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="AK1" s="24" t="s">
         <v>25</v>
@@ -1313,11 +1310,11 @@
         <v>26</v>
       </c>
       <c r="AM1" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="30" t="s">
         <v>27</v>
       </c>
       <c r="B2" s="26" t="s">
@@ -1333,7 +1330,7 @@
       <c r="AM2" s="5"/>
     </row>
     <row r="3" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="35"/>
+      <c r="A3" s="31"/>
       <c r="B3" s="26" t="s">
         <v>29</v>
       </c>
@@ -1346,7 +1343,7 @@
       <c r="AM3" s="5"/>
     </row>
     <row r="4" spans="1:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="35"/>
+      <c r="A4" s="31"/>
       <c r="B4" s="26" t="s">
         <v>30</v>
       </c>
@@ -1360,7 +1357,7 @@
       <c r="AM4" s="5"/>
     </row>
     <row r="5" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="35"/>
+      <c r="A5" s="31"/>
       <c r="B5" s="26" t="s">
         <v>31</v>
       </c>
@@ -1373,7 +1370,7 @@
       <c r="AM5" s="5"/>
     </row>
     <row r="6" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="35"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="26" t="s">
         <v>32</v>
       </c>
@@ -1386,7 +1383,7 @@
       <c r="AM6" s="5"/>
     </row>
     <row r="7" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="35"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="26" t="s">
         <v>33</v>
       </c>
@@ -1399,7 +1396,7 @@
       <c r="AM7" s="5"/>
     </row>
     <row r="8" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="35"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="26" t="s">
         <v>34</v>
       </c>
@@ -1412,7 +1409,7 @@
       <c r="AM8" s="5"/>
     </row>
     <row r="9" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="35"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="26" t="s">
         <v>35</v>
       </c>
@@ -1425,7 +1422,7 @@
       <c r="AM9" s="5"/>
     </row>
     <row r="10" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="35"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="26" t="s">
         <v>36</v>
       </c>
@@ -1438,12 +1435,12 @@
       <c r="AM10" s="5"/>
     </row>
     <row r="11" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="36"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="27" t="s">
         <v>0</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D11" s="2">
         <f t="shared" ref="D11:X11" si="0">SUM(D2:D10)</f>
@@ -1591,7 +1588,7 @@
       </c>
     </row>
     <row r="12" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="33" t="s">
         <v>37</v>
       </c>
       <c r="B12" s="26" t="s">
@@ -1606,7 +1603,7 @@
       <c r="AM12" s="5"/>
     </row>
     <row r="13" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="35"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="26" t="s">
         <v>29</v>
       </c>
@@ -1619,7 +1616,7 @@
       <c r="AM13" s="5"/>
     </row>
     <row r="14" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="35"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="26" t="s">
         <v>30</v>
       </c>
@@ -1632,7 +1629,7 @@
       <c r="AM14" s="5"/>
     </row>
     <row r="15" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="35"/>
+      <c r="A15" s="31"/>
       <c r="B15" s="26" t="s">
         <v>31</v>
       </c>
@@ -1645,7 +1642,7 @@
       <c r="AM15" s="5"/>
     </row>
     <row r="16" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="35"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="26" t="s">
         <v>32</v>
       </c>
@@ -1658,7 +1655,7 @@
       <c r="AM16" s="5"/>
     </row>
     <row r="17" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="35"/>
+      <c r="A17" s="31"/>
       <c r="B17" s="26" t="s">
         <v>33</v>
       </c>
@@ -1671,7 +1668,7 @@
       <c r="AM17" s="5"/>
     </row>
     <row r="18" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="35"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="26" t="s">
         <v>34</v>
       </c>
@@ -1684,7 +1681,7 @@
       <c r="AM18" s="5"/>
     </row>
     <row r="19" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="35"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="26" t="s">
         <v>35</v>
       </c>
@@ -1697,7 +1694,7 @@
       <c r="AM19" s="5"/>
     </row>
     <row r="20" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="35"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="26" t="s">
         <v>36</v>
       </c>
@@ -1710,12 +1707,12 @@
       <c r="AM20" s="5"/>
     </row>
     <row r="21" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="36"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="28" t="s">
         <v>0</v>
       </c>
       <c r="C21" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D21" s="3">
         <f t="shared" ref="D21:X21" si="2">SUM(D12:D20)</f>
@@ -1866,9 +1863,7 @@
       <c r="A22" s="4"/>
     </row>
     <row r="29" spans="1:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C29" s="6" t="s">
-        <v>49</v>
-      </c>
+      <c r="C29" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1915,13 +1910,13 @@
         <v>38</v>
       </c>
       <c r="E1" s="29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F1" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="G1" s="29" t="s">
         <v>78</v>
-      </c>
-      <c r="G1" s="29" t="s">
-        <v>79</v>
       </c>
       <c r="H1" s="29" t="s">
         <v>7</v>
@@ -1939,13 +1934,13 @@
         <v>41</v>
       </c>
       <c r="M1" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="N1" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="N1" s="29" t="s">
+      <c r="O1" s="29" t="s">
         <v>82</v>
-      </c>
-      <c r="O1" s="29" t="s">
-        <v>83</v>
       </c>
       <c r="P1" s="29" t="s">
         <v>42</v>
@@ -1954,40 +1949,40 @@
         <v>43</v>
       </c>
       <c r="R1" s="29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S1" s="29" t="s">
         <v>45</v>
       </c>
       <c r="T1" s="29" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="U1" s="29" t="s">
         <v>46</v>
       </c>
       <c r="V1" s="29" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="W1" s="29" t="s">
+        <v>89</v>
+      </c>
+      <c r="X1" s="29" t="s">
         <v>90</v>
-      </c>
-      <c r="X1" s="29" t="s">
-        <v>91</v>
       </c>
       <c r="Y1" s="29" t="s">
         <v>47</v>
       </c>
       <c r="Z1" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="AA1" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="AA1" s="29" t="s">
+      <c r="AB1" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="AB1" s="29" t="s">
+      <c r="AC1" s="29" t="s">
         <v>86</v>
-      </c>
-      <c r="AC1" s="29" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="12.75" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
removed personal metadata from sheet template
</commit_message>
<xml_diff>
--- a/Stat_Template_DO_NOT_REMOVE.xlsx
+++ b/Stat_Template_DO_NOT_REMOVE.xlsx
@@ -2,15 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\super\OneDrive\Documents\Python Projects\SluggersStatTracker\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59FA2570-89A2-4970-9A18-5A8ED2D0626D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00CE50B6-55DA-43BA-B60C-062F5C4333A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1950" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game Info" sheetId="3" r:id="rId1"/>
@@ -611,6 +606,18 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
@@ -622,18 +629,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -865,18 +860,18 @@
   </cols>
   <sheetData>
     <row r="9" spans="9:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="L9" s="34"/>
-      <c r="M9" s="34"/>
-      <c r="N9" s="34"/>
-      <c r="O9" s="34"/>
-      <c r="P9" s="34"/>
+      <c r="L9" s="30"/>
+      <c r="M9" s="30"/>
+      <c r="N9" s="30"/>
+      <c r="O9" s="30"/>
+      <c r="P9" s="30"/>
     </row>
     <row r="10" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="L10" s="35"/>
-      <c r="M10" s="35"/>
-      <c r="N10" s="35"/>
-      <c r="O10" s="35"/>
-      <c r="P10" s="35"/>
+      <c r="L10" s="31"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
+      <c r="O10" s="31"/>
+      <c r="P10" s="31"/>
     </row>
     <row r="11" spans="9:19" ht="59.25" x14ac:dyDescent="0.75">
       <c r="J11" s="14"/>
@@ -891,83 +886,83 @@
       </c>
     </row>
     <row r="12" spans="9:19" ht="40.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="I12" s="37" t="s">
+      <c r="I12" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="J12" s="37"/>
-      <c r="K12" s="37"/>
-      <c r="L12" s="37"/>
-      <c r="P12" s="37" t="s">
+      <c r="J12" s="33"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="33"/>
+      <c r="P12" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="Q12" s="37"/>
-      <c r="R12" s="37"/>
-      <c r="S12" s="37"/>
+      <c r="Q12" s="33"/>
+      <c r="R12" s="33"/>
+      <c r="S12" s="33"/>
     </row>
     <row r="13" spans="9:19" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="I13" s="36" t="s">
+      <c r="I13" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="J13" s="36"/>
-      <c r="K13" s="36"/>
-      <c r="L13" s="36"/>
-      <c r="P13" s="36" t="s">
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="32"/>
+      <c r="P13" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="Q13" s="36"/>
-      <c r="R13" s="36"/>
-      <c r="S13" s="36"/>
+      <c r="Q13" s="32"/>
+      <c r="R13" s="32"/>
+      <c r="S13" s="32"/>
     </row>
     <row r="14" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="I14" s="35" t="s">
+      <c r="I14" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="J14" s="35"/>
-      <c r="K14" s="35"/>
-      <c r="L14" s="35"/>
-      <c r="M14" s="35"/>
-      <c r="N14" s="35"/>
-      <c r="O14" s="35"/>
-      <c r="P14" s="35"/>
-      <c r="Q14" s="35"/>
-      <c r="R14" s="35"/>
-      <c r="S14" s="35"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="31"/>
+      <c r="N14" s="31"/>
+      <c r="O14" s="31"/>
+      <c r="P14" s="31"/>
+      <c r="Q14" s="31"/>
+      <c r="R14" s="31"/>
+      <c r="S14" s="31"/>
     </row>
     <row r="15" spans="9:19" ht="18" x14ac:dyDescent="0.25">
       <c r="I15" s="18"/>
       <c r="J15" s="18"/>
       <c r="K15" s="18"/>
       <c r="L15" s="18"/>
-      <c r="M15" s="35" t="s">
+      <c r="M15" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="N15" s="35"/>
-      <c r="O15" s="35"/>
+      <c r="N15" s="31"/>
+      <c r="O15" s="31"/>
       <c r="P15" s="18"/>
       <c r="Q15" s="18"/>
       <c r="R15" s="18"/>
       <c r="S15" s="18"/>
     </row>
     <row r="16" spans="9:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="M16" s="35" t="s">
+      <c r="M16" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="N16" s="35"/>
-      <c r="O16" s="35"/>
+      <c r="N16" s="31"/>
+      <c r="O16" s="31"/>
     </row>
     <row r="17" spans="10:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="M17" s="35" t="s">
+      <c r="M17" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="N17" s="35"/>
-      <c r="O17" s="35"/>
+      <c r="N17" s="31"/>
+      <c r="O17" s="31"/>
     </row>
     <row r="18" spans="10:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="M18" s="35" t="s">
+      <c r="M18" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="N18" s="34"/>
-      <c r="O18" s="34"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="30"/>
     </row>
     <row r="19" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J19" s="19" t="s">
@@ -1110,12 +1105,12 @@
       </c>
     </row>
     <row r="29" spans="10:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="M29" s="35" t="s">
+      <c r="M29" s="31" t="s">
         <v>88</v>
       </c>
-      <c r="N29" s="35"/>
-      <c r="O29" s="35"/>
-      <c r="P29" s="35"/>
+      <c r="N29" s="31"/>
+      <c r="O29" s="31"/>
+      <c r="P29" s="31"/>
     </row>
     <row r="31" spans="10:18" ht="15" x14ac:dyDescent="0.2">
       <c r="J31" s="17" t="s">
@@ -1144,6 +1139,7 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1314,7 +1310,7 @@
       </c>
     </row>
     <row r="2" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="34" t="s">
         <v>27</v>
       </c>
       <c r="B2" s="26" t="s">
@@ -1330,7 +1326,7 @@
       <c r="AM2" s="5"/>
     </row>
     <row r="3" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="31"/>
+      <c r="A3" s="35"/>
       <c r="B3" s="26" t="s">
         <v>29</v>
       </c>
@@ -1343,7 +1339,7 @@
       <c r="AM3" s="5"/>
     </row>
     <row r="4" spans="1:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="31"/>
+      <c r="A4" s="35"/>
       <c r="B4" s="26" t="s">
         <v>30</v>
       </c>
@@ -1357,7 +1353,7 @@
       <c r="AM4" s="5"/>
     </row>
     <row r="5" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="31"/>
+      <c r="A5" s="35"/>
       <c r="B5" s="26" t="s">
         <v>31</v>
       </c>
@@ -1370,7 +1366,7 @@
       <c r="AM5" s="5"/>
     </row>
     <row r="6" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="31"/>
+      <c r="A6" s="35"/>
       <c r="B6" s="26" t="s">
         <v>32</v>
       </c>
@@ -1383,7 +1379,7 @@
       <c r="AM6" s="5"/>
     </row>
     <row r="7" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="31"/>
+      <c r="A7" s="35"/>
       <c r="B7" s="26" t="s">
         <v>33</v>
       </c>
@@ -1396,7 +1392,7 @@
       <c r="AM7" s="5"/>
     </row>
     <row r="8" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="31"/>
+      <c r="A8" s="35"/>
       <c r="B8" s="26" t="s">
         <v>34</v>
       </c>
@@ -1409,7 +1405,7 @@
       <c r="AM8" s="5"/>
     </row>
     <row r="9" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="31"/>
+      <c r="A9" s="35"/>
       <c r="B9" s="26" t="s">
         <v>35</v>
       </c>
@@ -1422,7 +1418,7 @@
       <c r="AM9" s="5"/>
     </row>
     <row r="10" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="31"/>
+      <c r="A10" s="35"/>
       <c r="B10" s="26" t="s">
         <v>36</v>
       </c>
@@ -1435,7 +1431,7 @@
       <c r="AM10" s="5"/>
     </row>
     <row r="11" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="32"/>
+      <c r="A11" s="36"/>
       <c r="B11" s="27" t="s">
         <v>0</v>
       </c>
@@ -1588,7 +1584,7 @@
       </c>
     </row>
     <row r="12" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="37" t="s">
         <v>37</v>
       </c>
       <c r="B12" s="26" t="s">
@@ -1603,7 +1599,7 @@
       <c r="AM12" s="5"/>
     </row>
     <row r="13" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="31"/>
+      <c r="A13" s="35"/>
       <c r="B13" s="26" t="s">
         <v>29</v>
       </c>
@@ -1616,7 +1612,7 @@
       <c r="AM13" s="5"/>
     </row>
     <row r="14" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="31"/>
+      <c r="A14" s="35"/>
       <c r="B14" s="26" t="s">
         <v>30</v>
       </c>
@@ -1629,7 +1625,7 @@
       <c r="AM14" s="5"/>
     </row>
     <row r="15" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="31"/>
+      <c r="A15" s="35"/>
       <c r="B15" s="26" t="s">
         <v>31</v>
       </c>
@@ -1642,7 +1638,7 @@
       <c r="AM15" s="5"/>
     </row>
     <row r="16" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="31"/>
+      <c r="A16" s="35"/>
       <c r="B16" s="26" t="s">
         <v>32</v>
       </c>
@@ -1655,7 +1651,7 @@
       <c r="AM16" s="5"/>
     </row>
     <row r="17" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="31"/>
+      <c r="A17" s="35"/>
       <c r="B17" s="26" t="s">
         <v>33</v>
       </c>
@@ -1668,7 +1664,7 @@
       <c r="AM17" s="5"/>
     </row>
     <row r="18" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="31"/>
+      <c r="A18" s="35"/>
       <c r="B18" s="26" t="s">
         <v>34</v>
       </c>
@@ -1681,7 +1677,7 @@
       <c r="AM18" s="5"/>
     </row>
     <row r="19" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="31"/>
+      <c r="A19" s="35"/>
       <c r="B19" s="26" t="s">
         <v>35</v>
       </c>
@@ -1694,7 +1690,7 @@
       <c r="AM19" s="5"/>
     </row>
     <row r="20" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="31"/>
+      <c r="A20" s="35"/>
       <c r="B20" s="26" t="s">
         <v>36</v>
       </c>
@@ -1707,7 +1703,7 @@
       <c r="AM20" s="5"/>
     </row>
     <row r="21" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="32"/>
+      <c r="A21" s="36"/>
       <c r="B21" s="28" t="s">
         <v>0</v>
       </c>
@@ -1871,6 +1867,7 @@
     <mergeCell ref="A12:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2503,5 +2500,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add new batting stats and update team branding names. fixed HR classification issue. added new logs
</commit_message>
<xml_diff>
--- a/Stat_Template_DO_NOT_REMOVE.xlsx
+++ b/Stat_Template_DO_NOT_REMOVE.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00CE50B6-55DA-43BA-B60C-062F5C4333A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D53EAC7-2A2B-4BFD-A093-7E7F187CBAC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-1950" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game Info" sheetId="3" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="103">
   <si>
     <t>Team</t>
   </si>
@@ -327,6 +327,18 @@
   </si>
   <si>
     <t>Pickoff Attempts</t>
+  </si>
+  <si>
+    <t>Double Plays Hit Into</t>
+  </si>
+  <si>
+    <t>Triple Plays Hit Into</t>
+  </si>
+  <si>
+    <t>Buddy Jumps Hit Into</t>
+  </si>
+  <si>
+    <t>Star Swings</t>
   </si>
 </sst>
 </file>
@@ -1148,7 +1160,7 @@
   <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AM29"/>
+  <dimension ref="A1:AQ29"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5703125" bestFit="1" customWidth="1"/>
@@ -1171,26 +1183,28 @@
     <col min="20" max="20" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="10.85546875" customWidth="1"/>
-    <col min="23" max="23" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.42578125" customWidth="1"/>
-    <col min="25" max="25" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.5703125" customWidth="1"/>
-    <col min="28" max="28" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.42578125" customWidth="1"/>
-    <col min="30" max="30" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="14.28515625" customWidth="1"/>
-    <col min="33" max="33" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.140625" customWidth="1"/>
-    <col min="36" max="36" width="19.5703125" customWidth="1"/>
-    <col min="37" max="37" width="12" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8.85546875" customWidth="1"/>
+    <col min="23" max="25" width="20.5703125" customWidth="1"/>
+    <col min="26" max="26" width="13.5703125" customWidth="1"/>
+    <col min="27" max="27" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="10.42578125" customWidth="1"/>
+    <col min="29" max="29" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="8.5703125" customWidth="1"/>
+    <col min="32" max="32" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.42578125" customWidth="1"/>
+    <col min="34" max="34" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="14.28515625" customWidth="1"/>
+    <col min="37" max="37" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="19.140625" customWidth="1"/>
+    <col min="40" max="40" width="19.5703125" customWidth="1"/>
+    <col min="41" max="41" width="12" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="21" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:43" s="21" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -1258,58 +1272,70 @@
         <v>52</v>
       </c>
       <c r="W1" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="X1" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y1" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="Z1" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="AA1" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="X1" s="24" t="s">
+      <c r="AB1" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="Y1" s="24" t="s">
+      <c r="AC1" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="Z1" s="24" t="s">
+      <c r="AD1" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="AA1" s="24" t="s">
+      <c r="AE1" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="AB1" s="24" t="s">
+      <c r="AF1" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="AC1" s="24" t="s">
+      <c r="AG1" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="AD1" s="24" t="s">
+      <c r="AH1" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="AE1" s="24" t="s">
+      <c r="AI1" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="AF1" s="24" t="s">
+      <c r="AJ1" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="AG1" s="24" t="s">
+      <c r="AK1" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="AH1" s="24" t="s">
+      <c r="AL1" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="AI1" s="24" t="s">
+      <c r="AM1" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="AJ1" s="24" t="s">
+      <c r="AN1" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="AK1" s="24" t="s">
+      <c r="AO1" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="AL1" s="24" t="s">
+      <c r="AP1" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="AM1" s="25" t="s">
+      <c r="AQ1" s="25" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="34" t="s">
         <v>27</v>
       </c>
@@ -1318,119 +1344,119 @@
       </c>
       <c r="C2" s="21"/>
       <c r="F2" s="1"/>
-      <c r="Y2" s="8"/>
-      <c r="Z2" s="8"/>
-      <c r="AA2" s="8"/>
-      <c r="AB2" s="8"/>
       <c r="AC2" s="8"/>
-      <c r="AM2" s="5"/>
-    </row>
-    <row r="3" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD2" s="8"/>
+      <c r="AE2" s="8"/>
+      <c r="AF2" s="8"/>
+      <c r="AG2" s="8"/>
+      <c r="AQ2" s="5"/>
+    </row>
+    <row r="3" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="35"/>
       <c r="B3" s="26" t="s">
         <v>29</v>
       </c>
       <c r="C3" s="21"/>
-      <c r="Y3" s="8"/>
-      <c r="Z3" s="8"/>
-      <c r="AA3" s="8"/>
-      <c r="AB3" s="8"/>
       <c r="AC3" s="8"/>
-      <c r="AM3" s="5"/>
-    </row>
-    <row r="4" spans="1:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AD3" s="8"/>
+      <c r="AE3" s="8"/>
+      <c r="AF3" s="8"/>
+      <c r="AG3" s="8"/>
+      <c r="AQ3" s="5"/>
+    </row>
+    <row r="4" spans="1:43" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="35"/>
       <c r="B4" s="26" t="s">
         <v>30</v>
       </c>
       <c r="C4" s="21"/>
       <c r="M4" s="1"/>
-      <c r="Y4" s="8"/>
-      <c r="Z4" s="8"/>
-      <c r="AA4" s="8"/>
-      <c r="AB4" s="8"/>
       <c r="AC4" s="8"/>
-      <c r="AM4" s="5"/>
-    </row>
-    <row r="5" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD4" s="8"/>
+      <c r="AE4" s="8"/>
+      <c r="AF4" s="8"/>
+      <c r="AG4" s="8"/>
+      <c r="AQ4" s="5"/>
+    </row>
+    <row r="5" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="35"/>
       <c r="B5" s="26" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="21"/>
-      <c r="Y5" s="8"/>
-      <c r="Z5" s="8"/>
-      <c r="AA5" s="8"/>
-      <c r="AB5" s="8"/>
       <c r="AC5" s="8"/>
-      <c r="AM5" s="5"/>
-    </row>
-    <row r="6" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD5" s="8"/>
+      <c r="AE5" s="8"/>
+      <c r="AF5" s="8"/>
+      <c r="AG5" s="8"/>
+      <c r="AQ5" s="5"/>
+    </row>
+    <row r="6" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="35"/>
       <c r="B6" s="26" t="s">
         <v>32</v>
       </c>
       <c r="C6" s="21"/>
-      <c r="Y6" s="8"/>
-      <c r="Z6" s="8"/>
-      <c r="AA6" s="8"/>
-      <c r="AB6" s="8"/>
       <c r="AC6" s="8"/>
-      <c r="AM6" s="5"/>
-    </row>
-    <row r="7" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD6" s="8"/>
+      <c r="AE6" s="8"/>
+      <c r="AF6" s="8"/>
+      <c r="AG6" s="8"/>
+      <c r="AQ6" s="5"/>
+    </row>
+    <row r="7" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="35"/>
       <c r="B7" s="26" t="s">
         <v>33</v>
       </c>
       <c r="C7" s="21"/>
-      <c r="Y7" s="8"/>
-      <c r="Z7" s="8"/>
-      <c r="AA7" s="8"/>
-      <c r="AB7" s="8"/>
       <c r="AC7" s="8"/>
-      <c r="AM7" s="5"/>
-    </row>
-    <row r="8" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD7" s="8"/>
+      <c r="AE7" s="8"/>
+      <c r="AF7" s="8"/>
+      <c r="AG7" s="8"/>
+      <c r="AQ7" s="5"/>
+    </row>
+    <row r="8" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="35"/>
       <c r="B8" s="26" t="s">
         <v>34</v>
       </c>
       <c r="C8" s="21"/>
-      <c r="Y8" s="8"/>
-      <c r="Z8" s="8"/>
-      <c r="AA8" s="8"/>
-      <c r="AB8" s="8"/>
       <c r="AC8" s="8"/>
-      <c r="AM8" s="5"/>
-    </row>
-    <row r="9" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD8" s="8"/>
+      <c r="AE8" s="8"/>
+      <c r="AF8" s="8"/>
+      <c r="AG8" s="8"/>
+      <c r="AQ8" s="5"/>
+    </row>
+    <row r="9" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="35"/>
       <c r="B9" s="26" t="s">
         <v>35</v>
       </c>
       <c r="C9" s="21"/>
-      <c r="Y9" s="8"/>
-      <c r="Z9" s="8"/>
-      <c r="AA9" s="8"/>
-      <c r="AB9" s="8"/>
       <c r="AC9" s="8"/>
-      <c r="AM9" s="5"/>
-    </row>
-    <row r="10" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD9" s="8"/>
+      <c r="AE9" s="8"/>
+      <c r="AF9" s="8"/>
+      <c r="AG9" s="8"/>
+      <c r="AQ9" s="5"/>
+    </row>
+    <row r="10" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="35"/>
       <c r="B10" s="26" t="s">
         <v>36</v>
       </c>
       <c r="C10" s="21"/>
-      <c r="Y10" s="8"/>
-      <c r="Z10" s="8"/>
-      <c r="AA10" s="8"/>
-      <c r="AB10" s="8"/>
       <c r="AC10" s="8"/>
-      <c r="AM10" s="5"/>
-    </row>
-    <row r="11" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD10" s="8"/>
+      <c r="AE10" s="8"/>
+      <c r="AF10" s="8"/>
+      <c r="AG10" s="8"/>
+      <c r="AQ10" s="5"/>
+    </row>
+    <row r="11" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="36"/>
       <c r="B11" s="27" t="s">
         <v>0</v>
@@ -1439,7 +1465,7 @@
         <v>51</v>
       </c>
       <c r="D11" s="2">
-        <f t="shared" ref="D11:X11" si="0">SUM(D2:D10)</f>
+        <f t="shared" ref="D11:AB11" si="0">SUM(D2:D10)</f>
         <v>0</v>
       </c>
       <c r="E11" s="2">
@@ -1522,68 +1548,84 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="Y11" s="9">
-        <f>IFERROR(AVERAGE(Y2:Y10), 0)</f>
-        <v>0</v>
-      </c>
-      <c r="Z11" s="9">
-        <f>IFERROR(AVERAGE(Z2:Z10), 0)</f>
-        <v>0</v>
-      </c>
-      <c r="AA11" s="9">
-        <f>IFERROR(AVERAGE(AA2:AA10), 0)</f>
-        <v>0</v>
-      </c>
-      <c r="AB11" s="9">
-        <f>IFERROR(AVERAGE(AB2:AB10), 0)</f>
+      <c r="Y11" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Z11" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AA11" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AB11" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AC11" s="9">
         <f>IFERROR(AVERAGE(AC2:AC10), 0)</f>
         <v>0</v>
       </c>
-      <c r="AD11" s="2">
-        <f t="shared" ref="AD11:AM11" si="1">SUM(AD2:AD10)</f>
-        <v>0</v>
-      </c>
-      <c r="AE11" s="2">
+      <c r="AD11" s="9">
+        <f>IFERROR(AVERAGE(AD2:AD10), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE11" s="9">
+        <f>IFERROR(AVERAGE(AE2:AE10), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="AF11" s="9">
+        <f>IFERROR(AVERAGE(AF2:AF10), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="AG11" s="9">
+        <f>IFERROR(AVERAGE(AG2:AG10), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="AH11" s="2">
+        <f t="shared" ref="AH11:AQ11" si="1">SUM(AH2:AH10)</f>
+        <v>0</v>
+      </c>
+      <c r="AI11" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AF11" s="2">
+      <c r="AJ11" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AG11" s="2">
+      <c r="AK11" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AH11" s="2">
-        <f>SUM(AH2:AH10)</f>
-        <v>0</v>
-      </c>
-      <c r="AI11" s="2">
-        <f>SUM(AI2:AI10)</f>
-        <v>0</v>
-      </c>
-      <c r="AJ11" s="2">
-        <f>SUM(AJ2:AJ10)</f>
-        <v>0</v>
-      </c>
-      <c r="AK11" s="2">
-        <f>SUM(AK2:AK10)</f>
-        <v>0</v>
-      </c>
       <c r="AL11" s="2">
+        <f>SUM(AL2:AL10)</f>
+        <v>0</v>
+      </c>
+      <c r="AM11" s="2">
+        <f>SUM(AM2:AM10)</f>
+        <v>0</v>
+      </c>
+      <c r="AN11" s="2">
+        <f>SUM(AN2:AN10)</f>
+        <v>0</v>
+      </c>
+      <c r="AO11" s="2">
+        <f>SUM(AO2:AO10)</f>
+        <v>0</v>
+      </c>
+      <c r="AP11" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AM11" s="2">
+      <c r="AQ11" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="37" t="s">
         <v>37</v>
       </c>
@@ -1591,118 +1633,118 @@
         <v>28</v>
       </c>
       <c r="C12" s="21"/>
-      <c r="Y12" s="8"/>
-      <c r="Z12" s="8"/>
-      <c r="AA12" s="8"/>
-      <c r="AB12" s="8"/>
       <c r="AC12" s="8"/>
-      <c r="AM12" s="5"/>
-    </row>
-    <row r="13" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD12" s="8"/>
+      <c r="AE12" s="8"/>
+      <c r="AF12" s="8"/>
+      <c r="AG12" s="8"/>
+      <c r="AQ12" s="5"/>
+    </row>
+    <row r="13" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="35"/>
       <c r="B13" s="26" t="s">
         <v>29</v>
       </c>
       <c r="C13" s="21"/>
-      <c r="Y13" s="8"/>
-      <c r="Z13" s="8"/>
-      <c r="AA13" s="8"/>
-      <c r="AB13" s="8"/>
       <c r="AC13" s="8"/>
-      <c r="AM13" s="5"/>
-    </row>
-    <row r="14" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD13" s="8"/>
+      <c r="AE13" s="8"/>
+      <c r="AF13" s="8"/>
+      <c r="AG13" s="8"/>
+      <c r="AQ13" s="5"/>
+    </row>
+    <row r="14" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="35"/>
       <c r="B14" s="26" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="21"/>
-      <c r="Y14" s="8"/>
-      <c r="Z14" s="8"/>
-      <c r="AA14" s="8"/>
-      <c r="AB14" s="8"/>
       <c r="AC14" s="8"/>
-      <c r="AM14" s="5"/>
-    </row>
-    <row r="15" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD14" s="8"/>
+      <c r="AE14" s="8"/>
+      <c r="AF14" s="8"/>
+      <c r="AG14" s="8"/>
+      <c r="AQ14" s="5"/>
+    </row>
+    <row r="15" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="35"/>
       <c r="B15" s="26" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="21"/>
-      <c r="Y15" s="8"/>
-      <c r="Z15" s="8"/>
-      <c r="AA15" s="8"/>
-      <c r="AB15" s="8"/>
       <c r="AC15" s="8"/>
-      <c r="AM15" s="5"/>
-    </row>
-    <row r="16" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD15" s="8"/>
+      <c r="AE15" s="8"/>
+      <c r="AF15" s="8"/>
+      <c r="AG15" s="8"/>
+      <c r="AQ15" s="5"/>
+    </row>
+    <row r="16" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="35"/>
       <c r="B16" s="26" t="s">
         <v>32</v>
       </c>
       <c r="C16" s="21"/>
-      <c r="Y16" s="8"/>
-      <c r="Z16" s="8"/>
-      <c r="AA16" s="8"/>
-      <c r="AB16" s="8"/>
       <c r="AC16" s="8"/>
-      <c r="AM16" s="5"/>
-    </row>
-    <row r="17" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD16" s="8"/>
+      <c r="AE16" s="8"/>
+      <c r="AF16" s="8"/>
+      <c r="AG16" s="8"/>
+      <c r="AQ16" s="5"/>
+    </row>
+    <row r="17" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="35"/>
       <c r="B17" s="26" t="s">
         <v>33</v>
       </c>
       <c r="C17" s="21"/>
-      <c r="Y17" s="8"/>
-      <c r="Z17" s="8"/>
-      <c r="AA17" s="8"/>
-      <c r="AB17" s="8"/>
       <c r="AC17" s="8"/>
-      <c r="AM17" s="5"/>
-    </row>
-    <row r="18" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD17" s="8"/>
+      <c r="AE17" s="8"/>
+      <c r="AF17" s="8"/>
+      <c r="AG17" s="8"/>
+      <c r="AQ17" s="5"/>
+    </row>
+    <row r="18" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="35"/>
       <c r="B18" s="26" t="s">
         <v>34</v>
       </c>
       <c r="C18" s="21"/>
-      <c r="Y18" s="8"/>
-      <c r="Z18" s="8"/>
-      <c r="AA18" s="8"/>
-      <c r="AB18" s="8"/>
       <c r="AC18" s="8"/>
-      <c r="AM18" s="5"/>
-    </row>
-    <row r="19" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD18" s="8"/>
+      <c r="AE18" s="8"/>
+      <c r="AF18" s="8"/>
+      <c r="AG18" s="8"/>
+      <c r="AQ18" s="5"/>
+    </row>
+    <row r="19" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="35"/>
       <c r="B19" s="26" t="s">
         <v>35</v>
       </c>
       <c r="C19" s="21"/>
-      <c r="Y19" s="8"/>
-      <c r="Z19" s="8"/>
-      <c r="AA19" s="8"/>
-      <c r="AB19" s="8"/>
       <c r="AC19" s="8"/>
-      <c r="AM19" s="5"/>
-    </row>
-    <row r="20" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD19" s="8"/>
+      <c r="AE19" s="8"/>
+      <c r="AF19" s="8"/>
+      <c r="AG19" s="8"/>
+      <c r="AQ19" s="5"/>
+    </row>
+    <row r="20" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="35"/>
       <c r="B20" s="26" t="s">
         <v>36</v>
       </c>
       <c r="C20" s="21"/>
-      <c r="Y20" s="8"/>
-      <c r="Z20" s="8"/>
-      <c r="AA20" s="8"/>
-      <c r="AB20" s="8"/>
       <c r="AC20" s="8"/>
-      <c r="AM20" s="5"/>
-    </row>
-    <row r="21" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AD20" s="8"/>
+      <c r="AE20" s="8"/>
+      <c r="AF20" s="8"/>
+      <c r="AG20" s="8"/>
+      <c r="AQ20" s="5"/>
+    </row>
+    <row r="21" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21" s="36"/>
       <c r="B21" s="28" t="s">
         <v>0</v>
@@ -1711,7 +1753,7 @@
         <v>51</v>
       </c>
       <c r="D21" s="3">
-        <f t="shared" ref="D21:X21" si="2">SUM(D12:D20)</f>
+        <f t="shared" ref="D21:AB21" si="2">SUM(D12:D20)</f>
         <v>0</v>
       </c>
       <c r="E21" s="3">
@@ -1794,44 +1836,44 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Y21" s="10">
-        <f>IFERROR(AVERAGE(Y12:Y20), 0)</f>
-        <v>0</v>
-      </c>
-      <c r="Z21" s="10">
-        <f>IFERROR(AVERAGE(Z12:Z20), 0)</f>
-        <v>0</v>
-      </c>
-      <c r="AA21" s="10">
-        <f>IFERROR(AVERAGE(AA12:AA20), 0)</f>
-        <v>0</v>
-      </c>
-      <c r="AB21" s="10">
-        <f>IFERROR(AVERAGE(AB12:AB20), 0)</f>
+      <c r="Y21" s="3">
+        <f>SUM(Y12:Y20)</f>
+        <v>0</v>
+      </c>
+      <c r="Z21" s="3">
+        <f>SUM(Z12:Z20)</f>
+        <v>0</v>
+      </c>
+      <c r="AA21" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AB21" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AC21" s="10">
         <f>IFERROR(AVERAGE(AC12:AC20), 0)</f>
         <v>0</v>
       </c>
-      <c r="AD21" s="3">
-        <f t="shared" ref="AD21:AM21" si="3">SUM(AD12:AD20)</f>
-        <v>0</v>
-      </c>
-      <c r="AE21" s="3">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AF21" s="3">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AG21" s="3">
-        <f t="shared" si="3"/>
+      <c r="AD21" s="10">
+        <f>IFERROR(AVERAGE(AD12:AD20), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE21" s="10">
+        <f>IFERROR(AVERAGE(AE12:AE20), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="AF21" s="10">
+        <f>IFERROR(AVERAGE(AF12:AF20), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="AG21" s="10">
+        <f>IFERROR(AVERAGE(AG12:AG20), 0)</f>
         <v>0</v>
       </c>
       <c r="AH21" s="3">
-        <f>SUM(AH12:AH20)</f>
+        <f t="shared" ref="AH21:AQ21" si="3">SUM(AH12:AH20)</f>
         <v>0</v>
       </c>
       <c r="AI21" s="3">
@@ -1847,18 +1889,34 @@
         <v>0</v>
       </c>
       <c r="AL21" s="3">
-        <f t="shared" si="3"/>
+        <f>SUM(AL12:AL20)</f>
         <v>0</v>
       </c>
       <c r="AM21" s="3">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:39" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="AN21" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AO21" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AP21" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AQ21" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:43" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22" s="4"/>
     </row>
-    <row r="29" spans="1:39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:43" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C29" s="6"/>
     </row>
   </sheetData>

</xml_diff>